<commit_message>
added systme based socring for past predictions
</commit_message>
<xml_diff>
--- a/stock_data.xlsx
+++ b/stock_data.xlsx
@@ -513,16 +513,16 @@
         <v>45902</v>
       </c>
       <c r="B4" t="n">
-        <v>633.8644298326893</v>
+        <v>633.8644906037873</v>
       </c>
       <c r="C4" t="n">
-        <v>636.8373685858147</v>
+        <v>636.8374296419402</v>
       </c>
       <c r="D4" t="n">
-        <v>631.2991262066306</v>
+        <v>631.2991867317828</v>
       </c>
       <c r="E4" t="n">
-        <v>636.61865234375</v>
+        <v>636.6187133789062</v>
       </c>
       <c r="F4" t="n">
         <v>81983500</v>
@@ -553,16 +553,16 @@
         <v>45904</v>
       </c>
       <c r="B6" t="n">
-        <v>640.7449431803722</v>
+        <v>640.7450037735979</v>
       </c>
       <c r="C6" t="n">
-        <v>645.4480098993379</v>
+        <v>645.4480709373178</v>
       </c>
       <c r="D6" t="n">
-        <v>639.8401594892221</v>
+        <v>639.8402199968853</v>
       </c>
       <c r="E6" t="n">
-        <v>645.4181518554688</v>
+        <v>645.418212890625</v>
       </c>
       <c r="F6" t="n">
         <v>65219200</v>
@@ -593,16 +593,16 @@
         <v>45908</v>
       </c>
       <c r="B8" t="n">
-        <v>644.9209975333657</v>
+        <v>644.9210585487652</v>
       </c>
       <c r="C8" t="n">
-        <v>646.1340715853498</v>
+        <v>646.1341327155172</v>
       </c>
       <c r="D8" t="n">
-        <v>643.5389099622073</v>
+        <v>643.5389708468488</v>
       </c>
       <c r="E8" t="n">
-        <v>645.1298217773438</v>
+        <v>645.1298828125</v>
       </c>
       <c r="F8" t="n">
         <v>63133100</v>
@@ -633,16 +633,16 @@
         <v>45910</v>
       </c>
       <c r="B10" t="n">
-        <v>649.8925329397852</v>
+        <v>649.8924717726807</v>
       </c>
       <c r="C10" t="n">
-        <v>650.8172220560821</v>
+        <v>650.817160801947</v>
       </c>
       <c r="D10" t="n">
-        <v>646.9195940128865</v>
+        <v>646.9195331255914</v>
       </c>
       <c r="E10" t="n">
-        <v>648.4906005859375</v>
+        <v>648.4905395507812</v>
       </c>
       <c r="F10" t="n">
         <v>78034500</v>
@@ -673,16 +673,16 @@
         <v>45912</v>
       </c>
       <c r="B12" t="n">
-        <v>653.8498075653706</v>
+        <v>653.8497465125743</v>
       </c>
       <c r="C12" t="n">
-        <v>655.3512060315065</v>
+        <v>655.3511448385181</v>
       </c>
       <c r="D12" t="n">
-        <v>653.1538480823614</v>
+        <v>653.1537870945498</v>
       </c>
       <c r="E12" t="n">
-        <v>653.660888671875</v>
+        <v>653.6608276367188</v>
       </c>
       <c r="F12" t="n">
         <v>72780100</v>
@@ -753,16 +753,16 @@
         <v>45918</v>
       </c>
       <c r="B16" t="n">
-        <v>658.1153912564865</v>
+        <v>658.1153302554297</v>
       </c>
       <c r="C16" t="n">
-        <v>661.0982828700095</v>
+        <v>661.098221592467</v>
       </c>
       <c r="D16" t="n">
-        <v>656.5046346401509</v>
+        <v>656.504573788396</v>
       </c>
       <c r="E16" t="n">
-        <v>658.4832763671875</v>
+        <v>658.4832153320312</v>
       </c>
       <c r="F16" t="n">
         <v>90459200</v>
@@ -2885,7 +2885,7 @@
         <v>689.4299926757812</v>
       </c>
       <c r="F122" t="n">
-        <v>99952100</v>
+        <v>100034000</v>
       </c>
     </row>
     <row r="123">
@@ -2899,13 +2899,13 @@
         <v>690</v>
       </c>
       <c r="D123" t="n">
-        <v>680.3709716796875</v>
+        <v>680.3699951171875</v>
       </c>
       <c r="E123" t="n">
-        <v>682.9299926757812</v>
+        <v>682.3900146484375</v>
       </c>
       <c r="F123" t="n">
-        <v>48215603</v>
+        <v>90421900</v>
       </c>
     </row>
   </sheetData>
@@ -3039,16 +3039,16 @@
         <v>45904</v>
       </c>
       <c r="B6" t="n">
-        <v>237.996365667052</v>
+        <v>237.9963808412042</v>
       </c>
       <c r="C6" t="n">
-        <v>239.4436041167336</v>
+        <v>239.4436193831587</v>
       </c>
       <c r="D6" t="n">
-        <v>236.2896273284533</v>
+        <v>236.2896423937874</v>
       </c>
       <c r="E6" t="n">
-        <v>239.3238372802734</v>
+        <v>239.3238525390625</v>
       </c>
       <c r="F6" t="n">
         <v>47549400</v>
@@ -3159,16 +3159,16 @@
         <v>45912</v>
       </c>
       <c r="B12" t="n">
-        <v>228.7839306820605</v>
+        <v>228.7839456246826</v>
       </c>
       <c r="C12" t="n">
-        <v>234.063860229386</v>
+        <v>234.0638755168574</v>
       </c>
       <c r="D12" t="n">
-        <v>228.584314210114</v>
+        <v>228.5843291396984</v>
       </c>
       <c r="E12" t="n">
-        <v>233.6247100830078</v>
+        <v>233.6247253417969</v>
       </c>
       <c r="F12" t="n">
         <v>55824200</v>
@@ -3479,16 +3479,16 @@
         <v>45936</v>
       </c>
       <c r="B28" t="n">
-        <v>257.499174775338</v>
+        <v>257.4992054474702</v>
       </c>
       <c r="C28" t="n">
-        <v>258.5771371766132</v>
+        <v>258.5771679771474</v>
       </c>
       <c r="D28" t="n">
-        <v>254.5647807987102</v>
+        <v>254.5648111213107</v>
       </c>
       <c r="E28" t="n">
-        <v>256.20166015625</v>
+        <v>256.2016906738281</v>
       </c>
       <c r="F28" t="n">
         <v>44664100</v>
@@ -3499,16 +3499,16 @@
         <v>45937</v>
       </c>
       <c r="B29" t="n">
-        <v>256.3214547692021</v>
+        <v>256.3214394907812</v>
       </c>
       <c r="C29" t="n">
-        <v>256.9103287268919</v>
+        <v>256.9103134133703</v>
       </c>
       <c r="D29" t="n">
-        <v>254.9440751402397</v>
+        <v>254.9440599439195</v>
       </c>
       <c r="E29" t="n">
-        <v>255.9920959472656</v>
+        <v>255.9920806884766</v>
       </c>
       <c r="F29" t="n">
         <v>31955800</v>
@@ -3519,16 +3519,16 @@
         <v>45938</v>
       </c>
       <c r="B30" t="n">
-        <v>256.0320127996357</v>
+        <v>256.0319824641754</v>
       </c>
       <c r="C30" t="n">
-        <v>258.0282082133661</v>
+        <v>258.0281776413904</v>
       </c>
       <c r="D30" t="n">
-        <v>255.6227890846779</v>
+        <v>255.6227587977037</v>
       </c>
       <c r="E30" t="n">
-        <v>257.569091796875</v>
+        <v>257.5690612792969</v>
       </c>
       <c r="F30" t="n">
         <v>36496900</v>
@@ -3619,16 +3619,16 @@
         <v>45945</v>
       </c>
       <c r="B35" t="n">
-        <v>249.0153854047813</v>
+        <v>249.0153701368122</v>
       </c>
       <c r="C35" t="n">
-        <v>251.3409547309234</v>
+        <v>251.3409393203658</v>
       </c>
       <c r="D35" t="n">
-        <v>246.9992239099275</v>
+        <v>246.999208765576</v>
       </c>
       <c r="E35" t="n">
-        <v>248.8656616210938</v>
+        <v>248.8656463623047</v>
       </c>
       <c r="F35" t="n">
         <v>33893600</v>
@@ -3639,16 +3639,16 @@
         <v>45946</v>
       </c>
       <c r="B36" t="n">
-        <v>247.7777444808599</v>
+        <v>247.7777291727393</v>
       </c>
       <c r="C36" t="n">
-        <v>248.5662349323926</v>
+        <v>248.5662195755578</v>
       </c>
       <c r="D36" t="n">
-        <v>244.6636846503341</v>
+        <v>244.6636695346054</v>
       </c>
       <c r="E36" t="n">
-        <v>246.9792633056641</v>
+        <v>246.979248046875</v>
       </c>
       <c r="F36" t="n">
         <v>39777000</v>
@@ -3699,16 +3699,16 @@
         <v>45951</v>
       </c>
       <c r="B39" t="n">
-        <v>261.3817895915523</v>
+        <v>261.3818200057694</v>
       </c>
       <c r="C39" t="n">
-        <v>264.7853058703715</v>
+        <v>264.7853366806196</v>
       </c>
       <c r="D39" t="n">
-        <v>261.3318664386604</v>
+        <v>261.3318968470685</v>
       </c>
       <c r="E39" t="n">
-        <v>262.2700805664062</v>
+        <v>262.2701110839844</v>
       </c>
       <c r="F39" t="n">
         <v>46695900</v>
@@ -3759,16 +3759,16 @@
         <v>45954</v>
       </c>
       <c r="B42" t="n">
-        <v>260.6931337605782</v>
+        <v>260.6931034322695</v>
       </c>
       <c r="C42" t="n">
-        <v>263.6275433572314</v>
+        <v>263.6275126875418</v>
       </c>
       <c r="D42" t="n">
-        <v>258.6869476899315</v>
+        <v>258.6869175950168</v>
       </c>
       <c r="E42" t="n">
-        <v>262.3200378417969</v>
+        <v>262.3200073242188</v>
       </c>
       <c r="F42" t="n">
         <v>38253700</v>
@@ -5371,7 +5371,7 @@
         <v>264.5799865722656</v>
       </c>
       <c r="F122" t="n">
-        <v>42044900</v>
+        <v>42070500</v>
       </c>
     </row>
     <row r="123">
@@ -5382,16 +5382,16 @@
         <v>263.489990234375</v>
       </c>
       <c r="C123" t="n">
-        <v>268.9299011230469</v>
+        <v>269.4299926757812</v>
       </c>
       <c r="D123" t="n">
-        <v>263.3810119628906</v>
+        <v>263.3800048828125</v>
       </c>
       <c r="E123" t="n">
-        <v>268.7040100097656</v>
+        <v>266.1799926757812</v>
       </c>
       <c r="F123" t="n">
-        <v>17837923</v>
+        <v>37266000</v>
       </c>
     </row>
   </sheetData>
@@ -7857,7 +7857,7 @@
         <v>397.2300109863281</v>
       </c>
       <c r="F122" t="n">
-        <v>33960000</v>
+        <v>34015200</v>
       </c>
     </row>
     <row r="123">
@@ -7865,19 +7865,19 @@
         <v>46076</v>
       </c>
       <c r="B123" t="n">
-        <v>395.1900024414062</v>
+        <v>395</v>
       </c>
       <c r="C123" t="n">
-        <v>395.3099975585938</v>
+        <v>395.3599853515625</v>
       </c>
       <c r="D123" t="n">
-        <v>385.1000061035156</v>
+        <v>383.1000061035156</v>
       </c>
       <c r="E123" t="n">
-        <v>387.0549926757812</v>
+        <v>384.4700012207031</v>
       </c>
       <c r="F123" t="n">
-        <v>24476560</v>
+        <v>43133000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added background prediction updates, as well as constant api calls for 1000/hour
</commit_message>
<xml_diff>
--- a/stock_data.xlsx
+++ b/stock_data.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SPY" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AAPL" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSFT" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AMZN" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,16 +514,16 @@
         <v>45931</v>
       </c>
       <c r="B4" t="n">
-        <v>659.4152702620313</v>
+        <v>659.4153308150761</v>
       </c>
       <c r="C4" t="n">
-        <v>665.5801794564833</v>
+        <v>665.5802405756418</v>
       </c>
       <c r="D4" t="n">
-        <v>659.3059076216911</v>
+        <v>659.3059681646932</v>
       </c>
       <c r="E4" t="n">
-        <v>664.6654052734375</v>
+        <v>664.6654663085938</v>
       </c>
       <c r="F4" t="n">
         <v>72545400</v>
@@ -713,16 +714,16 @@
         <v>45945</v>
       </c>
       <c r="B14" t="n">
-        <v>663.0446129876665</v>
+        <v>663.0446741742268</v>
       </c>
       <c r="C14" t="n">
-        <v>666.4352795829697</v>
+        <v>666.4353410824248</v>
       </c>
       <c r="D14" t="n">
-        <v>655.1992699391986</v>
+        <v>655.1993304017814</v>
       </c>
       <c r="E14" t="n">
-        <v>661.4039306640625</v>
+        <v>661.4039916992188</v>
       </c>
       <c r="F14" t="n">
         <v>81702600</v>
@@ -733,16 +734,16 @@
         <v>45946</v>
       </c>
       <c r="B15" t="n">
-        <v>663.0445999065358</v>
+        <v>663.0446615126489</v>
       </c>
       <c r="C15" t="n">
-        <v>664.9239136533134</v>
+        <v>664.9239754340409</v>
       </c>
       <c r="D15" t="n">
-        <v>653.3895542222015</v>
+        <v>653.3896149312258</v>
       </c>
       <c r="E15" t="n">
-        <v>656.8995971679688</v>
+        <v>656.899658203125</v>
       </c>
       <c r="F15" t="n">
         <v>110563300</v>
@@ -793,16 +794,16 @@
         <v>45951</v>
       </c>
       <c r="B18" t="n">
-        <v>667.638493864759</v>
+        <v>667.6384328159621</v>
       </c>
       <c r="C18" t="n">
-        <v>669.1797060532549</v>
+        <v>669.1796448635298</v>
       </c>
       <c r="D18" t="n">
-        <v>666.1867381348511</v>
+        <v>666.1866772188026</v>
       </c>
       <c r="E18" t="n">
-        <v>667.4893188476562</v>
+        <v>667.4892578125</v>
       </c>
       <c r="F18" t="n">
         <v>56249000</v>
@@ -913,16 +914,16 @@
         <v>45959</v>
       </c>
       <c r="B24" t="n">
-        <v>684.8206562449755</v>
+        <v>684.8205950917289</v>
       </c>
       <c r="C24" t="n">
-        <v>685.795149064121</v>
+        <v>685.795087823854</v>
       </c>
       <c r="D24" t="n">
-        <v>679.0038013689816</v>
+        <v>679.0037407351697</v>
       </c>
       <c r="E24" t="n">
-        <v>683.4982299804688</v>
+        <v>683.4981689453125</v>
       </c>
       <c r="F24" t="n">
         <v>85657100</v>
@@ -933,16 +934,16 @@
         <v>45960</v>
       </c>
       <c r="B25" t="n">
-        <v>680.0279821977349</v>
+        <v>680.0279207971732</v>
       </c>
       <c r="C25" t="n">
-        <v>682.0564104652303</v>
+        <v>682.0563488815194</v>
       </c>
       <c r="D25" t="n">
-        <v>675.9810180664062</v>
+        <v>675.98095703125</v>
       </c>
       <c r="E25" t="n">
-        <v>675.9810180664062</v>
+        <v>675.98095703125</v>
       </c>
       <c r="F25" t="n">
         <v>76335800</v>
@@ -953,16 +954,16 @@
         <v>45961</v>
       </c>
       <c r="B26" t="n">
-        <v>681.1614116072222</v>
+        <v>681.1614729090464</v>
       </c>
       <c r="C26" t="n">
-        <v>681.2012239761448</v>
+        <v>681.2012852815519</v>
       </c>
       <c r="D26" t="n">
-        <v>675.3942622450203</v>
+        <v>675.3943230278239</v>
       </c>
       <c r="E26" t="n">
-        <v>678.1983032226562</v>
+        <v>678.1983642578125</v>
       </c>
       <c r="F26" t="n">
         <v>87164100</v>
@@ -1073,16 +1074,16 @@
         <v>45971</v>
       </c>
       <c r="B32" t="n">
-        <v>673.4056154266486</v>
+        <v>673.4056760856186</v>
       </c>
       <c r="C32" t="n">
-        <v>678.3176487268574</v>
+        <v>678.317709828293</v>
       </c>
       <c r="D32" t="n">
-        <v>671.2081667723378</v>
+        <v>671.2082272333661</v>
       </c>
       <c r="E32" t="n">
-        <v>677.5818481445312</v>
+        <v>677.5819091796875</v>
       </c>
       <c r="F32" t="n">
         <v>75842900</v>
@@ -1113,16 +1114,16 @@
         <v>45973</v>
       </c>
       <c r="B34" t="n">
-        <v>680.9129156193362</v>
+        <v>680.9128544582501</v>
       </c>
       <c r="C34" t="n">
-        <v>681.0819968300743</v>
+        <v>681.081935653801</v>
       </c>
       <c r="D34" t="n">
-        <v>677.0946904605516</v>
+        <v>677.0946296424269</v>
       </c>
       <c r="E34" t="n">
-        <v>679.5109252929688</v>
+        <v>679.5108642578125</v>
       </c>
       <c r="F34" t="n">
         <v>62312500</v>
@@ -1133,16 +1134,16 @@
         <v>45974</v>
       </c>
       <c r="B35" t="n">
-        <v>676.6472315164618</v>
+        <v>676.6471697129602</v>
       </c>
       <c r="C35" t="n">
-        <v>677.0051787486752</v>
+        <v>677.0051169124795</v>
       </c>
       <c r="D35" t="n">
-        <v>666.7237544337754</v>
+        <v>666.7236935366629</v>
       </c>
       <c r="E35" t="n">
-        <v>668.235107421875</v>
+        <v>668.2350463867188</v>
       </c>
       <c r="F35" t="n">
         <v>103457800</v>
@@ -1153,16 +1154,16 @@
         <v>45975</v>
       </c>
       <c r="B36" t="n">
-        <v>661.612768198211</v>
+        <v>661.6128286383953</v>
       </c>
       <c r="C36" t="n">
-        <v>671.8345335183507</v>
+        <v>671.8345948923219</v>
       </c>
       <c r="D36" t="n">
-        <v>659.5147291242073</v>
+        <v>659.5147893727298</v>
       </c>
       <c r="E36" t="n">
-        <v>668.1256713867188</v>
+        <v>668.125732421875</v>
       </c>
       <c r="F36" t="n">
         <v>96846700</v>
@@ -1193,16 +1194,16 @@
         <v>45979</v>
       </c>
       <c r="B38" t="n">
-        <v>658.3512953245886</v>
+        <v>658.351356546523</v>
       </c>
       <c r="C38" t="n">
-        <v>661.354216097308</v>
+        <v>661.3542775984923</v>
       </c>
       <c r="D38" t="n">
-        <v>652.146634691611</v>
+        <v>652.1466953365565</v>
       </c>
       <c r="E38" t="n">
-        <v>656.3427734375</v>
+        <v>656.3428344726562</v>
       </c>
       <c r="F38" t="n">
         <v>114467500</v>
@@ -1213,16 +1214,16 @@
         <v>45980</v>
       </c>
       <c r="B39" t="n">
-        <v>657.0388554539629</v>
+        <v>657.0389163187169</v>
       </c>
       <c r="C39" t="n">
-        <v>663.5617119214406</v>
+        <v>663.561773390439</v>
       </c>
       <c r="D39" t="n">
-        <v>655.0203196831769</v>
+        <v>655.020380360944</v>
       </c>
       <c r="E39" t="n">
-        <v>658.8783569335938</v>
+        <v>658.87841796875</v>
       </c>
       <c r="F39" t="n">
         <v>94703000</v>
@@ -1293,16 +1294,16 @@
         <v>45986</v>
       </c>
       <c r="B43" t="n">
-        <v>664.8444060411854</v>
+        <v>664.8443455838128</v>
       </c>
       <c r="C43" t="n">
-        <v>672.3815071629971</v>
+        <v>672.3814460202411</v>
       </c>
       <c r="D43" t="n">
-        <v>660.717877921785</v>
+        <v>660.7178178396566</v>
       </c>
       <c r="E43" t="n">
-        <v>671.1982421875</v>
+        <v>671.1981811523438</v>
       </c>
       <c r="F43" t="n">
         <v>81077100</v>
@@ -1353,16 +1354,16 @@
         <v>45992</v>
       </c>
       <c r="B46" t="n">
-        <v>674.9667014318244</v>
+        <v>674.9667623359846</v>
       </c>
       <c r="C46" t="n">
-        <v>679.1230277654502</v>
+        <v>679.1230890446475</v>
       </c>
       <c r="D46" t="n">
-        <v>674.8970904760725</v>
+        <v>674.8971513739515</v>
       </c>
       <c r="E46" t="n">
-        <v>676.41845703125</v>
+        <v>676.4185180664062</v>
       </c>
       <c r="F46" t="n">
         <v>61201200</v>
@@ -1473,16 +1474,16 @@
         <v>46000</v>
       </c>
       <c r="B52" t="n">
-        <v>679.2822138612034</v>
+        <v>679.2821528162136</v>
       </c>
       <c r="C52" t="n">
-        <v>681.5095218770947</v>
+        <v>681.5094606319436</v>
       </c>
       <c r="D52" t="n">
-        <v>678.7253868572307</v>
+        <v>678.7253258622812</v>
       </c>
       <c r="E52" t="n">
-        <v>679.1727905273438</v>
+        <v>679.1727294921875</v>
       </c>
       <c r="F52" t="n">
         <v>58310100</v>
@@ -1533,16 +1534,16 @@
         <v>46003</v>
       </c>
       <c r="B55" t="n">
-        <v>684.2737672143002</v>
+        <v>684.2737056052856</v>
       </c>
       <c r="C55" t="n">
-        <v>684.9797692517327</v>
+        <v>684.9797075791527</v>
       </c>
       <c r="D55" t="n">
-        <v>675.3247225627367</v>
+        <v>675.3246617594549</v>
       </c>
       <c r="E55" t="n">
-        <v>677.9000854492188</v>
+        <v>677.9000244140625</v>
       </c>
       <c r="F55" t="n">
         <v>113160300</v>
@@ -2946,6 +2947,26 @@
       </c>
       <c r="F125" t="n">
         <v>96353600</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="B126" t="n">
+        <v>642.5</v>
+      </c>
+      <c r="C126" t="n">
+        <v>642.6599731445312</v>
+      </c>
+      <c r="D126" t="n">
+        <v>638.3400268554688</v>
+      </c>
+      <c r="E126" t="n">
+        <v>639.47998046875</v>
+      </c>
+      <c r="F126" t="n">
+        <v>38597554</v>
       </c>
     </row>
   </sheetData>
@@ -2959,7 +2980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5472,6 +5493,26 @@
       </c>
       <c r="F125" t="n">
         <v>41702500</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="B126" t="n">
+        <v>253.9100036621094</v>
+      </c>
+      <c r="C126" t="n">
+        <v>255.4929962158203</v>
+      </c>
+      <c r="D126" t="n">
+        <v>251.8000030517578</v>
+      </c>
+      <c r="E126" t="n">
+        <v>252.3600006103516</v>
+      </c>
+      <c r="F126" t="n">
+        <v>17773290</v>
       </c>
     </row>
   </sheetData>
@@ -5485,7 +5526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8000,6 +8041,2572 @@
         <v>36719800</v>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="B126" t="n">
+        <v>362.0400085449219</v>
+      </c>
+      <c r="C126" t="n">
+        <v>362.4249877929688</v>
+      </c>
+      <c r="D126" t="n">
+        <v>356.5799865722656</v>
+      </c>
+      <c r="E126" t="n">
+        <v>360.2449951171875</v>
+      </c>
+      <c r="F126" t="n">
+        <v>16973651</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F126"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>45929</v>
+      </c>
+      <c r="B2" t="n">
+        <v>220.0800018310547</v>
+      </c>
+      <c r="C2" t="n">
+        <v>222.6000061035156</v>
+      </c>
+      <c r="D2" t="n">
+        <v>219.3000030517578</v>
+      </c>
+      <c r="E2" t="n">
+        <v>222.1699981689453</v>
+      </c>
+      <c r="F2" t="n">
+        <v>44259200</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>45930</v>
+      </c>
+      <c r="B3" t="n">
+        <v>222.0299987792969</v>
+      </c>
+      <c r="C3" t="n">
+        <v>222.2400054931641</v>
+      </c>
+      <c r="D3" t="n">
+        <v>217.8899993896484</v>
+      </c>
+      <c r="E3" t="n">
+        <v>219.5700073242188</v>
+      </c>
+      <c r="F3" t="n">
+        <v>48396400</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>45931</v>
+      </c>
+      <c r="B4" t="n">
+        <v>217.3600006103516</v>
+      </c>
+      <c r="C4" t="n">
+        <v>222.1499938964844</v>
+      </c>
+      <c r="D4" t="n">
+        <v>216.6100006103516</v>
+      </c>
+      <c r="E4" t="n">
+        <v>220.6300048828125</v>
+      </c>
+      <c r="F4" t="n">
+        <v>43933800</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>45932</v>
+      </c>
+      <c r="B5" t="n">
+        <v>221.0099945068359</v>
+      </c>
+      <c r="C5" t="n">
+        <v>222.8099975585938</v>
+      </c>
+      <c r="D5" t="n">
+        <v>218.9499969482422</v>
+      </c>
+      <c r="E5" t="n">
+        <v>222.4100036621094</v>
+      </c>
+      <c r="F5" t="n">
+        <v>41258600</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>45933</v>
+      </c>
+      <c r="B6" t="n">
+        <v>223.4400024414062</v>
+      </c>
+      <c r="C6" t="n">
+        <v>224.1999969482422</v>
+      </c>
+      <c r="D6" t="n">
+        <v>219.3399963378906</v>
+      </c>
+      <c r="E6" t="n">
+        <v>219.5099945068359</v>
+      </c>
+      <c r="F6" t="n">
+        <v>43639000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>45936</v>
+      </c>
+      <c r="B7" t="n">
+        <v>221</v>
+      </c>
+      <c r="C7" t="n">
+        <v>221.7299957275391</v>
+      </c>
+      <c r="D7" t="n">
+        <v>216.0299987792969</v>
+      </c>
+      <c r="E7" t="n">
+        <v>220.8999938964844</v>
+      </c>
+      <c r="F7" t="n">
+        <v>43690900</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>45937</v>
+      </c>
+      <c r="B8" t="n">
+        <v>220.8800048828125</v>
+      </c>
+      <c r="C8" t="n">
+        <v>222.8899993896484</v>
+      </c>
+      <c r="D8" t="n">
+        <v>220.1699981689453</v>
+      </c>
+      <c r="E8" t="n">
+        <v>221.7799987792969</v>
+      </c>
+      <c r="F8" t="n">
+        <v>31194700</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>45938</v>
+      </c>
+      <c r="B9" t="n">
+        <v>222.9199981689453</v>
+      </c>
+      <c r="C9" t="n">
+        <v>226.7299957275391</v>
+      </c>
+      <c r="D9" t="n">
+        <v>221.1900024414062</v>
+      </c>
+      <c r="E9" t="n">
+        <v>225.2200012207031</v>
+      </c>
+      <c r="F9" t="n">
+        <v>46686000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>45939</v>
+      </c>
+      <c r="B10" t="n">
+        <v>225</v>
+      </c>
+      <c r="C10" t="n">
+        <v>228.2100067138672</v>
+      </c>
+      <c r="D10" t="n">
+        <v>221.75</v>
+      </c>
+      <c r="E10" t="n">
+        <v>227.7400054931641</v>
+      </c>
+      <c r="F10" t="n">
+        <v>46412100</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>45940</v>
+      </c>
+      <c r="B11" t="n">
+        <v>226.2100067138672</v>
+      </c>
+      <c r="C11" t="n">
+        <v>228.25</v>
+      </c>
+      <c r="D11" t="n">
+        <v>216</v>
+      </c>
+      <c r="E11" t="n">
+        <v>216.3699951171875</v>
+      </c>
+      <c r="F11" t="n">
+        <v>72367500</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>45943</v>
+      </c>
+      <c r="B12" t="n">
+        <v>217.6999969482422</v>
+      </c>
+      <c r="C12" t="n">
+        <v>220.6799926757812</v>
+      </c>
+      <c r="D12" t="n">
+        <v>217.0399932861328</v>
+      </c>
+      <c r="E12" t="n">
+        <v>220.0700073242188</v>
+      </c>
+      <c r="F12" t="n">
+        <v>37809700</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>45944</v>
+      </c>
+      <c r="B13" t="n">
+        <v>215.5599975585938</v>
+      </c>
+      <c r="C13" t="n">
+        <v>219.3200073242188</v>
+      </c>
+      <c r="D13" t="n">
+        <v>212.6000061035156</v>
+      </c>
+      <c r="E13" t="n">
+        <v>216.3899993896484</v>
+      </c>
+      <c r="F13" t="n">
+        <v>45665600</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>45945</v>
+      </c>
+      <c r="B14" t="n">
+        <v>216.6199951171875</v>
+      </c>
+      <c r="C14" t="n">
+        <v>217.7100067138672</v>
+      </c>
+      <c r="D14" t="n">
+        <v>212.6600036621094</v>
+      </c>
+      <c r="E14" t="n">
+        <v>215.5700073242188</v>
+      </c>
+      <c r="F14" t="n">
+        <v>45909500</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>45946</v>
+      </c>
+      <c r="B15" t="n">
+        <v>215.6699981689453</v>
+      </c>
+      <c r="C15" t="n">
+        <v>218.5899963378906</v>
+      </c>
+      <c r="D15" t="n">
+        <v>212.8099975585938</v>
+      </c>
+      <c r="E15" t="n">
+        <v>214.4700012207031</v>
+      </c>
+      <c r="F15" t="n">
+        <v>42414600</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>45947</v>
+      </c>
+      <c r="B16" t="n">
+        <v>214.5599975585938</v>
+      </c>
+      <c r="C16" t="n">
+        <v>214.8000030517578</v>
+      </c>
+      <c r="D16" t="n">
+        <v>211.0299987792969</v>
+      </c>
+      <c r="E16" t="n">
+        <v>213.0399932861328</v>
+      </c>
+      <c r="F16" t="n">
+        <v>45986900</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>45950</v>
+      </c>
+      <c r="B17" t="n">
+        <v>213.8800048828125</v>
+      </c>
+      <c r="C17" t="n">
+        <v>216.6900024414062</v>
+      </c>
+      <c r="D17" t="n">
+        <v>213.5899963378906</v>
+      </c>
+      <c r="E17" t="n">
+        <v>216.4799957275391</v>
+      </c>
+      <c r="F17" t="n">
+        <v>38882800</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>45951</v>
+      </c>
+      <c r="B18" t="n">
+        <v>218.4299926757812</v>
+      </c>
+      <c r="C18" t="n">
+        <v>223.3200073242188</v>
+      </c>
+      <c r="D18" t="n">
+        <v>217.9900054931641</v>
+      </c>
+      <c r="E18" t="n">
+        <v>222.0299987792969</v>
+      </c>
+      <c r="F18" t="n">
+        <v>50494600</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>45952</v>
+      </c>
+      <c r="B19" t="n">
+        <v>219.3000030517578</v>
+      </c>
+      <c r="C19" t="n">
+        <v>220.0099945068359</v>
+      </c>
+      <c r="D19" t="n">
+        <v>216.5200042724609</v>
+      </c>
+      <c r="E19" t="n">
+        <v>217.9499969482422</v>
+      </c>
+      <c r="F19" t="n">
+        <v>44308500</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>45953</v>
+      </c>
+      <c r="B20" t="n">
+        <v>219</v>
+      </c>
+      <c r="C20" t="n">
+        <v>221.3000030517578</v>
+      </c>
+      <c r="D20" t="n">
+        <v>218.1799926757812</v>
+      </c>
+      <c r="E20" t="n">
+        <v>221.0899963378906</v>
+      </c>
+      <c r="F20" t="n">
+        <v>31540000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>45954</v>
+      </c>
+      <c r="B21" t="n">
+        <v>221.9700012207031</v>
+      </c>
+      <c r="C21" t="n">
+        <v>225.3999938964844</v>
+      </c>
+      <c r="D21" t="n">
+        <v>221.8999938964844</v>
+      </c>
+      <c r="E21" t="n">
+        <v>224.2100067138672</v>
+      </c>
+      <c r="F21" t="n">
+        <v>38685100</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>45957</v>
+      </c>
+      <c r="B22" t="n">
+        <v>227.6600036621094</v>
+      </c>
+      <c r="C22" t="n">
+        <v>228.3999938964844</v>
+      </c>
+      <c r="D22" t="n">
+        <v>225.5399932861328</v>
+      </c>
+      <c r="E22" t="n">
+        <v>226.9700012207031</v>
+      </c>
+      <c r="F22" t="n">
+        <v>38267000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>45958</v>
+      </c>
+      <c r="B23" t="n">
+        <v>228.2200012207031</v>
+      </c>
+      <c r="C23" t="n">
+        <v>231.4900054931641</v>
+      </c>
+      <c r="D23" t="n">
+        <v>226.2100067138672</v>
+      </c>
+      <c r="E23" t="n">
+        <v>229.25</v>
+      </c>
+      <c r="F23" t="n">
+        <v>47100000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>45959</v>
+      </c>
+      <c r="B24" t="n">
+        <v>231.6699981689453</v>
+      </c>
+      <c r="C24" t="n">
+        <v>232.8200073242188</v>
+      </c>
+      <c r="D24" t="n">
+        <v>227.7599945068359</v>
+      </c>
+      <c r="E24" t="n">
+        <v>230.3000030517578</v>
+      </c>
+      <c r="F24" t="n">
+        <v>52036200</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>45960</v>
+      </c>
+      <c r="B25" t="n">
+        <v>227.0599975585938</v>
+      </c>
+      <c r="C25" t="n">
+        <v>228.4400024414062</v>
+      </c>
+      <c r="D25" t="n">
+        <v>222.75</v>
+      </c>
+      <c r="E25" t="n">
+        <v>222.8600006103516</v>
+      </c>
+      <c r="F25" t="n">
+        <v>102252900</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>45961</v>
+      </c>
+      <c r="B26" t="n">
+        <v>250.1000061035156</v>
+      </c>
+      <c r="C26" t="n">
+        <v>250.5</v>
+      </c>
+      <c r="D26" t="n">
+        <v>243.9799957275391</v>
+      </c>
+      <c r="E26" t="n">
+        <v>244.2200012207031</v>
+      </c>
+      <c r="F26" t="n">
+        <v>166340800</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>45964</v>
+      </c>
+      <c r="B27" t="n">
+        <v>255.3600006103516</v>
+      </c>
+      <c r="C27" t="n">
+        <v>258.6000061035156</v>
+      </c>
+      <c r="D27" t="n">
+        <v>252.8999938964844</v>
+      </c>
+      <c r="E27" t="n">
+        <v>254</v>
+      </c>
+      <c r="F27" t="n">
+        <v>95997800</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>45965</v>
+      </c>
+      <c r="B28" t="n">
+        <v>250.3800048828125</v>
+      </c>
+      <c r="C28" t="n">
+        <v>257.010009765625</v>
+      </c>
+      <c r="D28" t="n">
+        <v>248.6600036621094</v>
+      </c>
+      <c r="E28" t="n">
+        <v>249.3200073242188</v>
+      </c>
+      <c r="F28" t="n">
+        <v>51546300</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>45966</v>
+      </c>
+      <c r="B29" t="n">
+        <v>249.0299987792969</v>
+      </c>
+      <c r="C29" t="n">
+        <v>251</v>
+      </c>
+      <c r="D29" t="n">
+        <v>246.1600036621094</v>
+      </c>
+      <c r="E29" t="n">
+        <v>250.1999969482422</v>
+      </c>
+      <c r="F29" t="n">
+        <v>40610700</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>45967</v>
+      </c>
+      <c r="B30" t="n">
+        <v>249.1600036621094</v>
+      </c>
+      <c r="C30" t="n">
+        <v>250.3800048828125</v>
+      </c>
+      <c r="D30" t="n">
+        <v>242.1699981689453</v>
+      </c>
+      <c r="E30" t="n">
+        <v>243.0399932861328</v>
+      </c>
+      <c r="F30" t="n">
+        <v>46004200</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>45968</v>
+      </c>
+      <c r="B31" t="n">
+        <v>242.8999938964844</v>
+      </c>
+      <c r="C31" t="n">
+        <v>244.8999938964844</v>
+      </c>
+      <c r="D31" t="n">
+        <v>238.4900054931641</v>
+      </c>
+      <c r="E31" t="n">
+        <v>244.4100036621094</v>
+      </c>
+      <c r="F31" t="n">
+        <v>46374300</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>45971</v>
+      </c>
+      <c r="B32" t="n">
+        <v>248.3399963378906</v>
+      </c>
+      <c r="C32" t="n">
+        <v>251.75</v>
+      </c>
+      <c r="D32" t="n">
+        <v>245.5899963378906</v>
+      </c>
+      <c r="E32" t="n">
+        <v>248.3999938964844</v>
+      </c>
+      <c r="F32" t="n">
+        <v>36476500</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>45972</v>
+      </c>
+      <c r="B33" t="n">
+        <v>248.4100036621094</v>
+      </c>
+      <c r="C33" t="n">
+        <v>249.75</v>
+      </c>
+      <c r="D33" t="n">
+        <v>247.2299957275391</v>
+      </c>
+      <c r="E33" t="n">
+        <v>249.1000061035156</v>
+      </c>
+      <c r="F33" t="n">
+        <v>23564100</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>45973</v>
+      </c>
+      <c r="B34" t="n">
+        <v>250.2400054931641</v>
+      </c>
+      <c r="C34" t="n">
+        <v>250.3699951171875</v>
+      </c>
+      <c r="D34" t="n">
+        <v>243.75</v>
+      </c>
+      <c r="E34" t="n">
+        <v>244.1999969482422</v>
+      </c>
+      <c r="F34" t="n">
+        <v>31190100</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>45974</v>
+      </c>
+      <c r="B35" t="n">
+        <v>243.0500030517578</v>
+      </c>
+      <c r="C35" t="n">
+        <v>243.75</v>
+      </c>
+      <c r="D35" t="n">
+        <v>236.5</v>
+      </c>
+      <c r="E35" t="n">
+        <v>237.5800018310547</v>
+      </c>
+      <c r="F35" t="n">
+        <v>41401700</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>45975</v>
+      </c>
+      <c r="B36" t="n">
+        <v>235.0599975585938</v>
+      </c>
+      <c r="C36" t="n">
+        <v>238.7299957275391</v>
+      </c>
+      <c r="D36" t="n">
+        <v>232.8899993896484</v>
+      </c>
+      <c r="E36" t="n">
+        <v>234.6900024414062</v>
+      </c>
+      <c r="F36" t="n">
+        <v>38956700</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>45978</v>
+      </c>
+      <c r="B37" t="n">
+        <v>233.25</v>
+      </c>
+      <c r="C37" t="n">
+        <v>234.6000061035156</v>
+      </c>
+      <c r="D37" t="n">
+        <v>229.1900024414062</v>
+      </c>
+      <c r="E37" t="n">
+        <v>232.8699951171875</v>
+      </c>
+      <c r="F37" t="n">
+        <v>59919000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>45979</v>
+      </c>
+      <c r="B38" t="n">
+        <v>228.1000061035156</v>
+      </c>
+      <c r="C38" t="n">
+        <v>230.1999969482422</v>
+      </c>
+      <c r="D38" t="n">
+        <v>222.4199981689453</v>
+      </c>
+      <c r="E38" t="n">
+        <v>222.5500030517578</v>
+      </c>
+      <c r="F38" t="n">
+        <v>60608400</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>45980</v>
+      </c>
+      <c r="B39" t="n">
+        <v>223.7400054931641</v>
+      </c>
+      <c r="C39" t="n">
+        <v>223.7400054931641</v>
+      </c>
+      <c r="D39" t="n">
+        <v>218.5200042724609</v>
+      </c>
+      <c r="E39" t="n">
+        <v>222.6900024414062</v>
+      </c>
+      <c r="F39" t="n">
+        <v>58335600</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>45981</v>
+      </c>
+      <c r="B40" t="n">
+        <v>227.0500030517578</v>
+      </c>
+      <c r="C40" t="n">
+        <v>227.4100036621094</v>
+      </c>
+      <c r="D40" t="n">
+        <v>216.7400054931641</v>
+      </c>
+      <c r="E40" t="n">
+        <v>217.1399993896484</v>
+      </c>
+      <c r="F40" t="n">
+        <v>50309000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>45982</v>
+      </c>
+      <c r="B41" t="n">
+        <v>216.3500061035156</v>
+      </c>
+      <c r="C41" t="n">
+        <v>222.2100067138672</v>
+      </c>
+      <c r="D41" t="n">
+        <v>215.1799926757812</v>
+      </c>
+      <c r="E41" t="n">
+        <v>220.6900024414062</v>
+      </c>
+      <c r="F41" t="n">
+        <v>68490500</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>45985</v>
+      </c>
+      <c r="B42" t="n">
+        <v>222.5599975585938</v>
+      </c>
+      <c r="C42" t="n">
+        <v>227.3300018310547</v>
+      </c>
+      <c r="D42" t="n">
+        <v>222.2700042724609</v>
+      </c>
+      <c r="E42" t="n">
+        <v>226.2799987792969</v>
+      </c>
+      <c r="F42" t="n">
+        <v>54318400</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>45986</v>
+      </c>
+      <c r="B43" t="n">
+        <v>226.3800048828125</v>
+      </c>
+      <c r="C43" t="n">
+        <v>230.5200042724609</v>
+      </c>
+      <c r="D43" t="n">
+        <v>223.8000030517578</v>
+      </c>
+      <c r="E43" t="n">
+        <v>229.6699981689453</v>
+      </c>
+      <c r="F43" t="n">
+        <v>39379300</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>45987</v>
+      </c>
+      <c r="B44" t="n">
+        <v>230.7400054931641</v>
+      </c>
+      <c r="C44" t="n">
+        <v>231.75</v>
+      </c>
+      <c r="D44" t="n">
+        <v>228.7700042724609</v>
+      </c>
+      <c r="E44" t="n">
+        <v>229.1600036621094</v>
+      </c>
+      <c r="F44" t="n">
+        <v>38497900</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>45989</v>
+      </c>
+      <c r="B45" t="n">
+        <v>231.2400054931641</v>
+      </c>
+      <c r="C45" t="n">
+        <v>233.2899932861328</v>
+      </c>
+      <c r="D45" t="n">
+        <v>230.2200012207031</v>
+      </c>
+      <c r="E45" t="n">
+        <v>233.2200012207031</v>
+      </c>
+      <c r="F45" t="n">
+        <v>20292300</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B46" t="n">
+        <v>233.2200012207031</v>
+      </c>
+      <c r="C46" t="n">
+        <v>235.8000030517578</v>
+      </c>
+      <c r="D46" t="n">
+        <v>232.25</v>
+      </c>
+      <c r="E46" t="n">
+        <v>233.8800048828125</v>
+      </c>
+      <c r="F46" t="n">
+        <v>42904000</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>45993</v>
+      </c>
+      <c r="B47" t="n">
+        <v>235.0099945068359</v>
+      </c>
+      <c r="C47" t="n">
+        <v>238.9700012207031</v>
+      </c>
+      <c r="D47" t="n">
+        <v>233.5500030517578</v>
+      </c>
+      <c r="E47" t="n">
+        <v>234.4199981689453</v>
+      </c>
+      <c r="F47" t="n">
+        <v>45785400</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>45994</v>
+      </c>
+      <c r="B48" t="n">
+        <v>233.3500061035156</v>
+      </c>
+      <c r="C48" t="n">
+        <v>233.3800048828125</v>
+      </c>
+      <c r="D48" t="n">
+        <v>230.6100006103516</v>
+      </c>
+      <c r="E48" t="n">
+        <v>232.3800048828125</v>
+      </c>
+      <c r="F48" t="n">
+        <v>35495100</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>45995</v>
+      </c>
+      <c r="B49" t="n">
+        <v>232.7700042724609</v>
+      </c>
+      <c r="C49" t="n">
+        <v>233.5</v>
+      </c>
+      <c r="D49" t="n">
+        <v>226.8000030517578</v>
+      </c>
+      <c r="E49" t="n">
+        <v>229.1100006103516</v>
+      </c>
+      <c r="F49" t="n">
+        <v>45683200</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>45996</v>
+      </c>
+      <c r="B50" t="n">
+        <v>230.3200073242188</v>
+      </c>
+      <c r="C50" t="n">
+        <v>231.2400054931641</v>
+      </c>
+      <c r="D50" t="n">
+        <v>228.5500030517578</v>
+      </c>
+      <c r="E50" t="n">
+        <v>229.5299987792969</v>
+      </c>
+      <c r="F50" t="n">
+        <v>33117400</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>45999</v>
+      </c>
+      <c r="B51" t="n">
+        <v>229.5899963378906</v>
+      </c>
+      <c r="C51" t="n">
+        <v>230.8300018310547</v>
+      </c>
+      <c r="D51" t="n">
+        <v>226.2700042724609</v>
+      </c>
+      <c r="E51" t="n">
+        <v>226.8899993896484</v>
+      </c>
+      <c r="F51" t="n">
+        <v>35019200</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46000</v>
+      </c>
+      <c r="B52" t="n">
+        <v>226.8399963378906</v>
+      </c>
+      <c r="C52" t="n">
+        <v>228.5700073242188</v>
+      </c>
+      <c r="D52" t="n">
+        <v>225.1100006103516</v>
+      </c>
+      <c r="E52" t="n">
+        <v>227.9199981689453</v>
+      </c>
+      <c r="F52" t="n">
+        <v>25841700</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46001</v>
+      </c>
+      <c r="B53" t="n">
+        <v>228.8099975585938</v>
+      </c>
+      <c r="C53" t="n">
+        <v>232.4199981689453</v>
+      </c>
+      <c r="D53" t="n">
+        <v>228.4600067138672</v>
+      </c>
+      <c r="E53" t="n">
+        <v>231.7799987792969</v>
+      </c>
+      <c r="F53" t="n">
+        <v>38790700</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46002</v>
+      </c>
+      <c r="B54" t="n">
+        <v>230.7100067138672</v>
+      </c>
+      <c r="C54" t="n">
+        <v>232.1100006103516</v>
+      </c>
+      <c r="D54" t="n">
+        <v>228.6900024414062</v>
+      </c>
+      <c r="E54" t="n">
+        <v>230.2799987792969</v>
+      </c>
+      <c r="F54" t="n">
+        <v>28249600</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46003</v>
+      </c>
+      <c r="B55" t="n">
+        <v>229.8699951171875</v>
+      </c>
+      <c r="C55" t="n">
+        <v>230.0800018310547</v>
+      </c>
+      <c r="D55" t="n">
+        <v>225.1199951171875</v>
+      </c>
+      <c r="E55" t="n">
+        <v>226.1900024414062</v>
+      </c>
+      <c r="F55" t="n">
+        <v>35639100</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46006</v>
+      </c>
+      <c r="B56" t="n">
+        <v>227.9299926757812</v>
+      </c>
+      <c r="C56" t="n">
+        <v>227.9299926757812</v>
+      </c>
+      <c r="D56" t="n">
+        <v>221.5</v>
+      </c>
+      <c r="E56" t="n">
+        <v>222.5399932861328</v>
+      </c>
+      <c r="F56" t="n">
+        <v>47286100</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46007</v>
+      </c>
+      <c r="B57" t="n">
+        <v>223.0399932861328</v>
+      </c>
+      <c r="C57" t="n">
+        <v>223.6600036621094</v>
+      </c>
+      <c r="D57" t="n">
+        <v>221.1300048828125</v>
+      </c>
+      <c r="E57" t="n">
+        <v>222.5599975585938</v>
+      </c>
+      <c r="F57" t="n">
+        <v>39298900</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46008</v>
+      </c>
+      <c r="B58" t="n">
+        <v>224.6600036621094</v>
+      </c>
+      <c r="C58" t="n">
+        <v>225.1900024414062</v>
+      </c>
+      <c r="D58" t="n">
+        <v>220.9900054931641</v>
+      </c>
+      <c r="E58" t="n">
+        <v>221.2700042724609</v>
+      </c>
+      <c r="F58" t="n">
+        <v>44034400</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B59" t="n">
+        <v>225.7100067138672</v>
+      </c>
+      <c r="C59" t="n">
+        <v>229.2299957275391</v>
+      </c>
+      <c r="D59" t="n">
+        <v>224.4100036621094</v>
+      </c>
+      <c r="E59" t="n">
+        <v>226.7599945068359</v>
+      </c>
+      <c r="F59" t="n">
+        <v>50272400</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46010</v>
+      </c>
+      <c r="B60" t="n">
+        <v>226.7599945068359</v>
+      </c>
+      <c r="C60" t="n">
+        <v>229.1300048828125</v>
+      </c>
+      <c r="D60" t="n">
+        <v>225.5800018310547</v>
+      </c>
+      <c r="E60" t="n">
+        <v>227.3500061035156</v>
+      </c>
+      <c r="F60" t="n">
+        <v>85544400</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46013</v>
+      </c>
+      <c r="B61" t="n">
+        <v>228.6100006103516</v>
+      </c>
+      <c r="C61" t="n">
+        <v>229.4799957275391</v>
+      </c>
+      <c r="D61" t="n">
+        <v>226.7100067138672</v>
+      </c>
+      <c r="E61" t="n">
+        <v>228.4299926757812</v>
+      </c>
+      <c r="F61" t="n">
+        <v>32261300</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46014</v>
+      </c>
+      <c r="B62" t="n">
+        <v>229.0599975585938</v>
+      </c>
+      <c r="C62" t="n">
+        <v>232.4499969482422</v>
+      </c>
+      <c r="D62" t="n">
+        <v>228.7299957275391</v>
+      </c>
+      <c r="E62" t="n">
+        <v>232.1399993896484</v>
+      </c>
+      <c r="F62" t="n">
+        <v>29230200</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46015</v>
+      </c>
+      <c r="B63" t="n">
+        <v>232.1300048828125</v>
+      </c>
+      <c r="C63" t="n">
+        <v>232.9499969482422</v>
+      </c>
+      <c r="D63" t="n">
+        <v>231.3300018310547</v>
+      </c>
+      <c r="E63" t="n">
+        <v>232.3800048828125</v>
+      </c>
+      <c r="F63" t="n">
+        <v>11420500</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46017</v>
+      </c>
+      <c r="B64" t="n">
+        <v>232.0399932861328</v>
+      </c>
+      <c r="C64" t="n">
+        <v>232.9900054931641</v>
+      </c>
+      <c r="D64" t="n">
+        <v>231.1799926757812</v>
+      </c>
+      <c r="E64" t="n">
+        <v>232.5200042724609</v>
+      </c>
+      <c r="F64" t="n">
+        <v>15994700</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46020</v>
+      </c>
+      <c r="B65" t="n">
+        <v>231.9400024414062</v>
+      </c>
+      <c r="C65" t="n">
+        <v>232.6000061035156</v>
+      </c>
+      <c r="D65" t="n">
+        <v>230.7700042724609</v>
+      </c>
+      <c r="E65" t="n">
+        <v>232.0700073242188</v>
+      </c>
+      <c r="F65" t="n">
+        <v>19797900</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46021</v>
+      </c>
+      <c r="B66" t="n">
+        <v>231.2100067138672</v>
+      </c>
+      <c r="C66" t="n">
+        <v>232.7700042724609</v>
+      </c>
+      <c r="D66" t="n">
+        <v>230.1999969482422</v>
+      </c>
+      <c r="E66" t="n">
+        <v>232.5299987792969</v>
+      </c>
+      <c r="F66" t="n">
+        <v>21910500</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46022</v>
+      </c>
+      <c r="B67" t="n">
+        <v>232.9100036621094</v>
+      </c>
+      <c r="C67" t="n">
+        <v>232.9900054931641</v>
+      </c>
+      <c r="D67" t="n">
+        <v>230.1199951171875</v>
+      </c>
+      <c r="E67" t="n">
+        <v>230.8200073242188</v>
+      </c>
+      <c r="F67" t="n">
+        <v>24383700</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46024</v>
+      </c>
+      <c r="B68" t="n">
+        <v>231.3399963378906</v>
+      </c>
+      <c r="C68" t="n">
+        <v>235.4600067138672</v>
+      </c>
+      <c r="D68" t="n">
+        <v>224.6999969482422</v>
+      </c>
+      <c r="E68" t="n">
+        <v>226.5</v>
+      </c>
+      <c r="F68" t="n">
+        <v>51456200</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B69" t="n">
+        <v>228.8399963378906</v>
+      </c>
+      <c r="C69" t="n">
+        <v>234</v>
+      </c>
+      <c r="D69" t="n">
+        <v>227.1799926757812</v>
+      </c>
+      <c r="E69" t="n">
+        <v>233.0599975585938</v>
+      </c>
+      <c r="F69" t="n">
+        <v>49733300</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46028</v>
+      </c>
+      <c r="B70" t="n">
+        <v>232.1000061035156</v>
+      </c>
+      <c r="C70" t="n">
+        <v>243.1799926757812</v>
+      </c>
+      <c r="D70" t="n">
+        <v>232.0700073242188</v>
+      </c>
+      <c r="E70" t="n">
+        <v>240.9299926757812</v>
+      </c>
+      <c r="F70" t="n">
+        <v>53764700</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46029</v>
+      </c>
+      <c r="B71" t="n">
+        <v>239.6100006103516</v>
+      </c>
+      <c r="C71" t="n">
+        <v>245.2899932861328</v>
+      </c>
+      <c r="D71" t="n">
+        <v>239.5200042724609</v>
+      </c>
+      <c r="E71" t="n">
+        <v>241.5599975585938</v>
+      </c>
+      <c r="F71" t="n">
+        <v>42236500</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46030</v>
+      </c>
+      <c r="B72" t="n">
+        <v>243.0599975585938</v>
+      </c>
+      <c r="C72" t="n">
+        <v>246.4100036621094</v>
+      </c>
+      <c r="D72" t="n">
+        <v>241.8800048828125</v>
+      </c>
+      <c r="E72" t="n">
+        <v>246.2899932861328</v>
+      </c>
+      <c r="F72" t="n">
+        <v>39509800</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46031</v>
+      </c>
+      <c r="B73" t="n">
+        <v>244.5700073242188</v>
+      </c>
+      <c r="C73" t="n">
+        <v>247.8600006103516</v>
+      </c>
+      <c r="D73" t="n">
+        <v>242.2400054931641</v>
+      </c>
+      <c r="E73" t="n">
+        <v>247.3800048828125</v>
+      </c>
+      <c r="F73" t="n">
+        <v>34560000</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="B74" t="n">
+        <v>246.7299957275391</v>
+      </c>
+      <c r="C74" t="n">
+        <v>248.9400024414062</v>
+      </c>
+      <c r="D74" t="n">
+        <v>245.9600067138672</v>
+      </c>
+      <c r="E74" t="n">
+        <v>246.4700012207031</v>
+      </c>
+      <c r="F74" t="n">
+        <v>35867800</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46035</v>
+      </c>
+      <c r="B75" t="n">
+        <v>246.5299987792969</v>
+      </c>
+      <c r="C75" t="n">
+        <v>247.6600036621094</v>
+      </c>
+      <c r="D75" t="n">
+        <v>240.25</v>
+      </c>
+      <c r="E75" t="n">
+        <v>242.6000061035156</v>
+      </c>
+      <c r="F75" t="n">
+        <v>38371800</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46036</v>
+      </c>
+      <c r="B76" t="n">
+        <v>241.1499938964844</v>
+      </c>
+      <c r="C76" t="n">
+        <v>241.2799987792969</v>
+      </c>
+      <c r="D76" t="n">
+        <v>236.2200012207031</v>
+      </c>
+      <c r="E76" t="n">
+        <v>236.6499938964844</v>
+      </c>
+      <c r="F76" t="n">
+        <v>41410600</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="B77" t="n">
+        <v>239.3099975585938</v>
+      </c>
+      <c r="C77" t="n">
+        <v>240.6499938964844</v>
+      </c>
+      <c r="D77" t="n">
+        <v>236.6300048828125</v>
+      </c>
+      <c r="E77" t="n">
+        <v>238.1799926757812</v>
+      </c>
+      <c r="F77" t="n">
+        <v>43003600</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46038</v>
+      </c>
+      <c r="B78" t="n">
+        <v>239.0899963378906</v>
+      </c>
+      <c r="C78" t="n">
+        <v>239.5700073242188</v>
+      </c>
+      <c r="D78" t="n">
+        <v>236.4100036621094</v>
+      </c>
+      <c r="E78" t="n">
+        <v>239.1199951171875</v>
+      </c>
+      <c r="F78" t="n">
+        <v>45888300</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="B79" t="n">
+        <v>233.7599945068359</v>
+      </c>
+      <c r="C79" t="n">
+        <v>235.0899963378906</v>
+      </c>
+      <c r="D79" t="n">
+        <v>229.3399963378906</v>
+      </c>
+      <c r="E79" t="n">
+        <v>231</v>
+      </c>
+      <c r="F79" t="n">
+        <v>47737900</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46043</v>
+      </c>
+      <c r="B80" t="n">
+        <v>231.0899963378906</v>
+      </c>
+      <c r="C80" t="n">
+        <v>232.3000030517578</v>
+      </c>
+      <c r="D80" t="n">
+        <v>226.8800048828125</v>
+      </c>
+      <c r="E80" t="n">
+        <v>231.3099975585938</v>
+      </c>
+      <c r="F80" t="n">
+        <v>47276100</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B81" t="n">
+        <v>234.0500030517578</v>
+      </c>
+      <c r="C81" t="n">
+        <v>235.7200012207031</v>
+      </c>
+      <c r="D81" t="n">
+        <v>230.8999938964844</v>
+      </c>
+      <c r="E81" t="n">
+        <v>234.3399963378906</v>
+      </c>
+      <c r="F81" t="n">
+        <v>31913300</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="B82" t="n">
+        <v>234.9600067138672</v>
+      </c>
+      <c r="C82" t="n">
+        <v>240.4499969482422</v>
+      </c>
+      <c r="D82" t="n">
+        <v>234.5700073242188</v>
+      </c>
+      <c r="E82" t="n">
+        <v>239.1600036621094</v>
+      </c>
+      <c r="F82" t="n">
+        <v>33778500</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46048</v>
+      </c>
+      <c r="B83" t="n">
+        <v>239.9799957275391</v>
+      </c>
+      <c r="C83" t="n">
+        <v>240.9499969482422</v>
+      </c>
+      <c r="D83" t="n">
+        <v>237.5399932861328</v>
+      </c>
+      <c r="E83" t="n">
+        <v>238.4199981689453</v>
+      </c>
+      <c r="F83" t="n">
+        <v>32825500</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46049</v>
+      </c>
+      <c r="B84" t="n">
+        <v>239.6900024414062</v>
+      </c>
+      <c r="C84" t="n">
+        <v>244.8800048828125</v>
+      </c>
+      <c r="D84" t="n">
+        <v>238.0800018310547</v>
+      </c>
+      <c r="E84" t="n">
+        <v>244.6799926757812</v>
+      </c>
+      <c r="F84" t="n">
+        <v>38029200</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="B85" t="n">
+        <v>246.3699951171875</v>
+      </c>
+      <c r="C85" t="n">
+        <v>247.7799987792969</v>
+      </c>
+      <c r="D85" t="n">
+        <v>241.5299987792969</v>
+      </c>
+      <c r="E85" t="n">
+        <v>243.0099945068359</v>
+      </c>
+      <c r="F85" t="n">
+        <v>40882700</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46051</v>
+      </c>
+      <c r="B86" t="n">
+        <v>242.8200073242188</v>
+      </c>
+      <c r="C86" t="n">
+        <v>243</v>
+      </c>
+      <c r="D86" t="n">
+        <v>236.7400054931641</v>
+      </c>
+      <c r="E86" t="n">
+        <v>241.7299957275391</v>
+      </c>
+      <c r="F86" t="n">
+        <v>47229600</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46052</v>
+      </c>
+      <c r="B87" t="n">
+        <v>239.8899993896484</v>
+      </c>
+      <c r="C87" t="n">
+        <v>243.3200073242188</v>
+      </c>
+      <c r="D87" t="n">
+        <v>237.6399993896484</v>
+      </c>
+      <c r="E87" t="n">
+        <v>239.3000030517578</v>
+      </c>
+      <c r="F87" t="n">
+        <v>46585000</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B88" t="n">
+        <v>238.3099975585938</v>
+      </c>
+      <c r="C88" t="n">
+        <v>245.6300048828125</v>
+      </c>
+      <c r="D88" t="n">
+        <v>238.1699981689453</v>
+      </c>
+      <c r="E88" t="n">
+        <v>242.9600067138672</v>
+      </c>
+      <c r="F88" t="n">
+        <v>37546100</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46056</v>
+      </c>
+      <c r="B89" t="n">
+        <v>244.9799957275391</v>
+      </c>
+      <c r="C89" t="n">
+        <v>246.3500061035156</v>
+      </c>
+      <c r="D89" t="n">
+        <v>235.4499969482422</v>
+      </c>
+      <c r="E89" t="n">
+        <v>238.6199951171875</v>
+      </c>
+      <c r="F89" t="n">
+        <v>53831300</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46057</v>
+      </c>
+      <c r="B90" t="n">
+        <v>238.8600006103516</v>
+      </c>
+      <c r="C90" t="n">
+        <v>238.8600006103516</v>
+      </c>
+      <c r="D90" t="n">
+        <v>231.8200073242188</v>
+      </c>
+      <c r="E90" t="n">
+        <v>232.9900054931641</v>
+      </c>
+      <c r="F90" t="n">
+        <v>51299900</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46058</v>
+      </c>
+      <c r="B91" t="n">
+        <v>224.9100036621094</v>
+      </c>
+      <c r="C91" t="n">
+        <v>226.3099975585938</v>
+      </c>
+      <c r="D91" t="n">
+        <v>220.3800048828125</v>
+      </c>
+      <c r="E91" t="n">
+        <v>222.6900024414062</v>
+      </c>
+      <c r="F91" t="n">
+        <v>103509200</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B92" t="n">
+        <v>202.6999969482422</v>
+      </c>
+      <c r="C92" t="n">
+        <v>211.4400024414062</v>
+      </c>
+      <c r="D92" t="n">
+        <v>200.3099975585938</v>
+      </c>
+      <c r="E92" t="n">
+        <v>210.3200073242188</v>
+      </c>
+      <c r="F92" t="n">
+        <v>179210900</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B93" t="n">
+        <v>208.9700012207031</v>
+      </c>
+      <c r="C93" t="n">
+        <v>212.8099975585938</v>
+      </c>
+      <c r="D93" t="n">
+        <v>203.3500061035156</v>
+      </c>
+      <c r="E93" t="n">
+        <v>208.7200012207031</v>
+      </c>
+      <c r="F93" t="n">
+        <v>91178400</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46063</v>
+      </c>
+      <c r="B94" t="n">
+        <v>208.8000030517578</v>
+      </c>
+      <c r="C94" t="n">
+        <v>212.6499938964844</v>
+      </c>
+      <c r="D94" t="n">
+        <v>206.4100036621094</v>
+      </c>
+      <c r="E94" t="n">
+        <v>206.9600067138672</v>
+      </c>
+      <c r="F94" t="n">
+        <v>67175000</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46064</v>
+      </c>
+      <c r="B95" t="n">
+        <v>208.0599975585938</v>
+      </c>
+      <c r="C95" t="n">
+        <v>208.5700073242188</v>
+      </c>
+      <c r="D95" t="n">
+        <v>202.4900054931641</v>
+      </c>
+      <c r="E95" t="n">
+        <v>204.0800018310547</v>
+      </c>
+      <c r="F95" t="n">
+        <v>65545500</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="B96" t="n">
+        <v>203.9600067138672</v>
+      </c>
+      <c r="C96" t="n">
+        <v>203.9600067138672</v>
+      </c>
+      <c r="D96" t="n">
+        <v>197.5599975585938</v>
+      </c>
+      <c r="E96" t="n">
+        <v>199.6000061035156</v>
+      </c>
+      <c r="F96" t="n">
+        <v>83975400</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46066</v>
+      </c>
+      <c r="B97" t="n">
+        <v>198.8800048828125</v>
+      </c>
+      <c r="C97" t="n">
+        <v>201.1600036621094</v>
+      </c>
+      <c r="D97" t="n">
+        <v>197.2799987792969</v>
+      </c>
+      <c r="E97" t="n">
+        <v>198.7899932861328</v>
+      </c>
+      <c r="F97" t="n">
+        <v>66321600</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="B98" t="n">
+        <v>198.1300048828125</v>
+      </c>
+      <c r="C98" t="n">
+        <v>201.7400054931641</v>
+      </c>
+      <c r="D98" t="n">
+        <v>196</v>
+      </c>
+      <c r="E98" t="n">
+        <v>201.1499938964844</v>
+      </c>
+      <c r="F98" t="n">
+        <v>69879200</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>46071</v>
+      </c>
+      <c r="B99" t="n">
+        <v>202.0700073242188</v>
+      </c>
+      <c r="C99" t="n">
+        <v>206.8600006103516</v>
+      </c>
+      <c r="D99" t="n">
+        <v>201.5099945068359</v>
+      </c>
+      <c r="E99" t="n">
+        <v>204.7899932861328</v>
+      </c>
+      <c r="F99" t="n">
+        <v>51003300</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>46072</v>
+      </c>
+      <c r="B100" t="n">
+        <v>203.8000030517578</v>
+      </c>
+      <c r="C100" t="n">
+        <v>205.6399993896484</v>
+      </c>
+      <c r="D100" t="n">
+        <v>202.8099975585938</v>
+      </c>
+      <c r="E100" t="n">
+        <v>204.8600006103516</v>
+      </c>
+      <c r="F100" t="n">
+        <v>35669600</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>46073</v>
+      </c>
+      <c r="B101" t="n">
+        <v>204.7599945068359</v>
+      </c>
+      <c r="C101" t="n">
+        <v>211.1699981689453</v>
+      </c>
+      <c r="D101" t="n">
+        <v>203.75</v>
+      </c>
+      <c r="E101" t="n">
+        <v>210.1100006103516</v>
+      </c>
+      <c r="F101" t="n">
+        <v>65881600</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>46076</v>
+      </c>
+      <c r="B102" t="n">
+        <v>208.1000061035156</v>
+      </c>
+      <c r="C102" t="n">
+        <v>208.4299926757812</v>
+      </c>
+      <c r="D102" t="n">
+        <v>203.1100006103516</v>
+      </c>
+      <c r="E102" t="n">
+        <v>205.2700042724609</v>
+      </c>
+      <c r="F102" t="n">
+        <v>53581500</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>46077</v>
+      </c>
+      <c r="B103" t="n">
+        <v>205.4700012207031</v>
+      </c>
+      <c r="C103" t="n">
+        <v>210.3600006103516</v>
+      </c>
+      <c r="D103" t="n">
+        <v>203.25</v>
+      </c>
+      <c r="E103" t="n">
+        <v>208.5599975585938</v>
+      </c>
+      <c r="F103" t="n">
+        <v>41137200</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="B104" t="n">
+        <v>210.4600067138672</v>
+      </c>
+      <c r="C104" t="n">
+        <v>211.5899963378906</v>
+      </c>
+      <c r="D104" t="n">
+        <v>208.9299926757812</v>
+      </c>
+      <c r="E104" t="n">
+        <v>210.6399993896484</v>
+      </c>
+      <c r="F104" t="n">
+        <v>41346400</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>46079</v>
+      </c>
+      <c r="B105" t="n">
+        <v>210.7299957275391</v>
+      </c>
+      <c r="C105" t="n">
+        <v>211.0500030517578</v>
+      </c>
+      <c r="D105" t="n">
+        <v>205.3500061035156</v>
+      </c>
+      <c r="E105" t="n">
+        <v>207.9199981689453</v>
+      </c>
+      <c r="F105" t="n">
+        <v>47756800</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>46080</v>
+      </c>
+      <c r="B106" t="n">
+        <v>206.8300018310547</v>
+      </c>
+      <c r="C106" t="n">
+        <v>210.3300018310547</v>
+      </c>
+      <c r="D106" t="n">
+        <v>205.1999969482422</v>
+      </c>
+      <c r="E106" t="n">
+        <v>210</v>
+      </c>
+      <c r="F106" t="n">
+        <v>57422800</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B107" t="n">
+        <v>204.5500030517578</v>
+      </c>
+      <c r="C107" t="n">
+        <v>209.7299957275391</v>
+      </c>
+      <c r="D107" t="n">
+        <v>203.4600067138672</v>
+      </c>
+      <c r="E107" t="n">
+        <v>208.3899993896484</v>
+      </c>
+      <c r="F107" t="n">
+        <v>46001000</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>46084</v>
+      </c>
+      <c r="B108" t="n">
+        <v>203.1000061035156</v>
+      </c>
+      <c r="C108" t="n">
+        <v>209.1799926757812</v>
+      </c>
+      <c r="D108" t="n">
+        <v>202.4799957275391</v>
+      </c>
+      <c r="E108" t="n">
+        <v>208.7299957275391</v>
+      </c>
+      <c r="F108" t="n">
+        <v>43184900</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>46085</v>
+      </c>
+      <c r="B109" t="n">
+        <v>210.4700012207031</v>
+      </c>
+      <c r="C109" t="n">
+        <v>217.5399932861328</v>
+      </c>
+      <c r="D109" t="n">
+        <v>210.1499938964844</v>
+      </c>
+      <c r="E109" t="n">
+        <v>216.8200073242188</v>
+      </c>
+      <c r="F109" t="n">
+        <v>54731100</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>46086</v>
+      </c>
+      <c r="B110" t="n">
+        <v>215.9799957275391</v>
+      </c>
+      <c r="C110" t="n">
+        <v>220.4700012207031</v>
+      </c>
+      <c r="D110" t="n">
+        <v>215.5899963378906</v>
+      </c>
+      <c r="E110" t="n">
+        <v>218.9400024414062</v>
+      </c>
+      <c r="F110" t="n">
+        <v>60943400</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>46087</v>
+      </c>
+      <c r="B111" t="n">
+        <v>214.9900054931641</v>
+      </c>
+      <c r="C111" t="n">
+        <v>217.3200073242188</v>
+      </c>
+      <c r="D111" t="n">
+        <v>212.5299987792969</v>
+      </c>
+      <c r="E111" t="n">
+        <v>213.2100067138672</v>
+      </c>
+      <c r="F111" t="n">
+        <v>51152700</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B112" t="n">
+        <v>210.4499969482422</v>
+      </c>
+      <c r="C112" t="n">
+        <v>213.8200073242188</v>
+      </c>
+      <c r="D112" t="n">
+        <v>207.1100006103516</v>
+      </c>
+      <c r="E112" t="n">
+        <v>213.4900054931641</v>
+      </c>
+      <c r="F112" t="n">
+        <v>54642900</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>46091</v>
+      </c>
+      <c r="B113" t="n">
+        <v>214.1900024414062</v>
+      </c>
+      <c r="C113" t="n">
+        <v>215.6499938964844</v>
+      </c>
+      <c r="D113" t="n">
+        <v>212.4299926757812</v>
+      </c>
+      <c r="E113" t="n">
+        <v>214.3300018310547</v>
+      </c>
+      <c r="F113" t="n">
+        <v>35678800</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>46092</v>
+      </c>
+      <c r="B114" t="n">
+        <v>215.7100067138672</v>
+      </c>
+      <c r="C114" t="n">
+        <v>217</v>
+      </c>
+      <c r="D114" t="n">
+        <v>211.3500061035156</v>
+      </c>
+      <c r="E114" t="n">
+        <v>212.6499938964844</v>
+      </c>
+      <c r="F114" t="n">
+        <v>34199300</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>46093</v>
+      </c>
+      <c r="B115" t="n">
+        <v>210.3899993896484</v>
+      </c>
+      <c r="C115" t="n">
+        <v>211.7100067138672</v>
+      </c>
+      <c r="D115" t="n">
+        <v>208.1499938964844</v>
+      </c>
+      <c r="E115" t="n">
+        <v>209.5299987792969</v>
+      </c>
+      <c r="F115" t="n">
+        <v>44349500</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>46094</v>
+      </c>
+      <c r="B116" t="n">
+        <v>209.6100006103516</v>
+      </c>
+      <c r="C116" t="n">
+        <v>210.5599975585938</v>
+      </c>
+      <c r="D116" t="n">
+        <v>206.2200012207031</v>
+      </c>
+      <c r="E116" t="n">
+        <v>207.6699981689453</v>
+      </c>
+      <c r="F116" t="n">
+        <v>35662100</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B117" t="n">
+        <v>208.3500061035156</v>
+      </c>
+      <c r="C117" t="n">
+        <v>212.7200012207031</v>
+      </c>
+      <c r="D117" t="n">
+        <v>207.4499969482422</v>
+      </c>
+      <c r="E117" t="n">
+        <v>211.7400054931641</v>
+      </c>
+      <c r="F117" t="n">
+        <v>42209300</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B118" t="n">
+        <v>212.8200073242188</v>
+      </c>
+      <c r="C118" t="n">
+        <v>215.6999969482422</v>
+      </c>
+      <c r="D118" t="n">
+        <v>212.4299926757812</v>
+      </c>
+      <c r="E118" t="n">
+        <v>215.1999969482422</v>
+      </c>
+      <c r="F118" t="n">
+        <v>44969900</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>46099</v>
+      </c>
+      <c r="B119" t="n">
+        <v>213.9299926757812</v>
+      </c>
+      <c r="C119" t="n">
+        <v>215.1399993896484</v>
+      </c>
+      <c r="D119" t="n">
+        <v>208.8300018310547</v>
+      </c>
+      <c r="E119" t="n">
+        <v>209.8699951171875</v>
+      </c>
+      <c r="F119" t="n">
+        <v>37846600</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="B120" t="n">
+        <v>207.0599975585938</v>
+      </c>
+      <c r="C120" t="n">
+        <v>209.1199951171875</v>
+      </c>
+      <c r="D120" t="n">
+        <v>206.0500030517578</v>
+      </c>
+      <c r="E120" t="n">
+        <v>208.7599945068359</v>
+      </c>
+      <c r="F120" t="n">
+        <v>36440600</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>46101</v>
+      </c>
+      <c r="B121" t="n">
+        <v>207.3999938964844</v>
+      </c>
+      <c r="C121" t="n">
+        <v>207.5399932861328</v>
+      </c>
+      <c r="D121" t="n">
+        <v>204.3200073242188</v>
+      </c>
+      <c r="E121" t="n">
+        <v>205.3699951171875</v>
+      </c>
+      <c r="F121" t="n">
+        <v>63694600</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>46104</v>
+      </c>
+      <c r="B122" t="n">
+        <v>209.7899932861328</v>
+      </c>
+      <c r="C122" t="n">
+        <v>212.8000030517578</v>
+      </c>
+      <c r="D122" t="n">
+        <v>209.5099945068359</v>
+      </c>
+      <c r="E122" t="n">
+        <v>210.1399993896484</v>
+      </c>
+      <c r="F122" t="n">
+        <v>44277400</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>46105</v>
+      </c>
+      <c r="B123" t="n">
+        <v>207.9499969482422</v>
+      </c>
+      <c r="C123" t="n">
+        <v>209.3500061035156</v>
+      </c>
+      <c r="D123" t="n">
+        <v>206.6399993896484</v>
+      </c>
+      <c r="E123" t="n">
+        <v>207.2400054931641</v>
+      </c>
+      <c r="F123" t="n">
+        <v>35351400</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>46106</v>
+      </c>
+      <c r="B124" t="n">
+        <v>211.5599975585938</v>
+      </c>
+      <c r="C124" t="n">
+        <v>213.0700073242188</v>
+      </c>
+      <c r="D124" t="n">
+        <v>209.8999938964844</v>
+      </c>
+      <c r="E124" t="n">
+        <v>211.7100067138672</v>
+      </c>
+      <c r="F124" t="n">
+        <v>36388800</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B125" t="n">
+        <v>210.6100006103516</v>
+      </c>
+      <c r="C125" t="n">
+        <v>212.8899993896484</v>
+      </c>
+      <c r="D125" t="n">
+        <v>207.1199951171875</v>
+      </c>
+      <c r="E125" t="n">
+        <v>207.5399932861328</v>
+      </c>
+      <c r="F125" t="n">
+        <v>46654700</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="B126" t="n">
+        <v>206.3249969482422</v>
+      </c>
+      <c r="C126" t="n">
+        <v>206.4199981689453</v>
+      </c>
+      <c r="D126" t="n">
+        <v>200.2700042724609</v>
+      </c>
+      <c r="E126" t="n">
+        <v>200.8399963378906</v>
+      </c>
+      <c r="F126" t="n">
+        <v>24190678</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added META to the predictions
</commit_message>
<xml_diff>
--- a/stock_data.xlsx
+++ b/stock_data.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AMZN" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSFT" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AAPL" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="META" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10373,4 +10374,2490 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F123"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>45940</v>
+      </c>
+      <c r="B2" t="n">
+        <v>729.6995938834806</v>
+      </c>
+      <c r="C2" t="n">
+        <v>734.0423674154782</v>
+      </c>
+      <c r="D2" t="n">
+        <v>703.333716456913</v>
+      </c>
+      <c r="E2" t="n">
+        <v>704.1223754882812</v>
+      </c>
+      <c r="F2" t="n">
+        <v>16980100</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>45943</v>
+      </c>
+      <c r="B3" t="n">
+        <v>711.8194939498104</v>
+      </c>
+      <c r="C3" t="n">
+        <v>718.7379155876384</v>
+      </c>
+      <c r="D3" t="n">
+        <v>706.4584651360833</v>
+      </c>
+      <c r="E3" t="n">
+        <v>714.5050048828125</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9251800</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>45944</v>
+      </c>
+      <c r="B4" t="n">
+        <v>706.598254382022</v>
+      </c>
+      <c r="C4" t="n">
+        <v>714.3552394376962</v>
+      </c>
+      <c r="D4" t="n">
+        <v>698.1623510959027</v>
+      </c>
+      <c r="E4" t="n">
+        <v>707.466796875</v>
+      </c>
+      <c r="F4" t="n">
+        <v>8829800</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>45945</v>
+      </c>
+      <c r="B5" t="n">
+        <v>715.8627565899488</v>
+      </c>
+      <c r="C5" t="n">
+        <v>722.6913629779451</v>
+      </c>
+      <c r="D5" t="n">
+        <v>708.3253746524584</v>
+      </c>
+      <c r="E5" t="n">
+        <v>716.3519287109375</v>
+      </c>
+      <c r="F5" t="n">
+        <v>10246800</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>45946</v>
+      </c>
+      <c r="B6" t="n">
+        <v>716.3519343648386</v>
+      </c>
+      <c r="C6" t="n">
+        <v>724.2786798244232</v>
+      </c>
+      <c r="D6" t="n">
+        <v>702.7047754671785</v>
+      </c>
+      <c r="E6" t="n">
+        <v>710.881103515625</v>
+      </c>
+      <c r="F6" t="n">
+        <v>9017000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>45947</v>
+      </c>
+      <c r="B7" t="n">
+        <v>705.8994251244851</v>
+      </c>
+      <c r="C7" t="n">
+        <v>717.3402516818879</v>
+      </c>
+      <c r="D7" t="n">
+        <v>704.9410060739878</v>
+      </c>
+      <c r="E7" t="n">
+        <v>715.7229614257812</v>
+      </c>
+      <c r="F7" t="n">
+        <v>12232400</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>45950</v>
+      </c>
+      <c r="B8" t="n">
+        <v>719.9858621042338</v>
+      </c>
+      <c r="C8" t="n">
+        <v>732.5448748734839</v>
+      </c>
+      <c r="D8" t="n">
+        <v>718.9775387090459</v>
+      </c>
+      <c r="E8" t="n">
+        <v>730.947509765625</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8900200</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>45951</v>
+      </c>
+      <c r="B9" t="n">
+        <v>734.7911237948646</v>
+      </c>
+      <c r="C9" t="n">
+        <v>737.2669635645257</v>
+      </c>
+      <c r="D9" t="n">
+        <v>727.5332426508437</v>
+      </c>
+      <c r="E9" t="n">
+        <v>732.0457153320312</v>
+      </c>
+      <c r="F9" t="n">
+        <v>7647300</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>45952</v>
+      </c>
+      <c r="B10" t="n">
+        <v>732.6047674176828</v>
+      </c>
+      <c r="C10" t="n">
+        <v>739.3634223567747</v>
+      </c>
+      <c r="D10" t="n">
+        <v>722.8211423130082</v>
+      </c>
+      <c r="E10" t="n">
+        <v>732.1854248046875</v>
+      </c>
+      <c r="F10" t="n">
+        <v>8734500</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>45953</v>
+      </c>
+      <c r="B11" t="n">
+        <v>733.4733185275871</v>
+      </c>
+      <c r="C11" t="n">
+        <v>741.170406509876</v>
+      </c>
+      <c r="D11" t="n">
+        <v>731.8759534115667</v>
+      </c>
+      <c r="E11" t="n">
+        <v>732.7744750976562</v>
+      </c>
+      <c r="F11" t="n">
+        <v>9856000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>45954</v>
+      </c>
+      <c r="B12" t="n">
+        <v>735.5598112729552</v>
+      </c>
+      <c r="C12" t="n">
+        <v>739.9724753796752</v>
+      </c>
+      <c r="D12" t="n">
+        <v>729.9292742962166</v>
+      </c>
+      <c r="E12" t="n">
+        <v>737.127197265625</v>
+      </c>
+      <c r="F12" t="n">
+        <v>9151300</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>45957</v>
+      </c>
+      <c r="B13" t="n">
+        <v>748.4781384032651</v>
+      </c>
+      <c r="C13" t="n">
+        <v>754.4881061640369</v>
+      </c>
+      <c r="D13" t="n">
+        <v>746.7610395763271</v>
+      </c>
+      <c r="E13" t="n">
+        <v>749.5663452148438</v>
+      </c>
+      <c r="F13" t="n">
+        <v>11321100</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>45958</v>
+      </c>
+      <c r="B14" t="n">
+        <v>751.3733793283152</v>
+      </c>
+      <c r="C14" t="n">
+        <v>757.1337649704751</v>
+      </c>
+      <c r="D14" t="n">
+        <v>744.2752651341964</v>
+      </c>
+      <c r="E14" t="n">
+        <v>750.1853637695312</v>
+      </c>
+      <c r="F14" t="n">
+        <v>12193800</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>45959</v>
+      </c>
+      <c r="B15" t="n">
+        <v>753.4897913670577</v>
+      </c>
+      <c r="C15" t="n">
+        <v>757.8924011644837</v>
+      </c>
+      <c r="D15" t="n">
+        <v>741.2702382858599</v>
+      </c>
+      <c r="E15" t="n">
+        <v>750.4149169921875</v>
+      </c>
+      <c r="F15" t="n">
+        <v>26818600</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>45960</v>
+      </c>
+      <c r="B16" t="n">
+        <v>668.0328178882455</v>
+      </c>
+      <c r="C16" t="n">
+        <v>679.8230975870755</v>
+      </c>
+      <c r="D16" t="n">
+        <v>649.0844652813799</v>
+      </c>
+      <c r="E16" t="n">
+        <v>665.3572387695312</v>
+      </c>
+      <c r="F16" t="n">
+        <v>88440100</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>45961</v>
+      </c>
+      <c r="B17" t="n">
+        <v>673.383812052831</v>
+      </c>
+      <c r="C17" t="n">
+        <v>673.7631824593219</v>
+      </c>
+      <c r="D17" t="n">
+        <v>644.4921293755289</v>
+      </c>
+      <c r="E17" t="n">
+        <v>647.2674560546875</v>
+      </c>
+      <c r="F17" t="n">
+        <v>56953200</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>45964</v>
+      </c>
+      <c r="B18" t="n">
+        <v>654.90470367213</v>
+      </c>
+      <c r="C18" t="n">
+        <v>658.2291607688485</v>
+      </c>
+      <c r="D18" t="n">
+        <v>635.1177890022415</v>
+      </c>
+      <c r="E18" t="n">
+        <v>636.645263671875</v>
+      </c>
+      <c r="F18" t="n">
+        <v>33003600</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>45965</v>
+      </c>
+      <c r="B19" t="n">
+        <v>626.9913515895119</v>
+      </c>
+      <c r="C19" t="n">
+        <v>640.6684891460408</v>
+      </c>
+      <c r="D19" t="n">
+        <v>624.9647727272926</v>
+      </c>
+      <c r="E19" t="n">
+        <v>626.2725830078125</v>
+      </c>
+      <c r="F19" t="n">
+        <v>27356600</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>45966</v>
+      </c>
+      <c r="B20" t="n">
+        <v>631.2542465797685</v>
+      </c>
+      <c r="C20" t="n">
+        <v>641.1576663615418</v>
+      </c>
+      <c r="D20" t="n">
+        <v>625.4938610947797</v>
+      </c>
+      <c r="E20" t="n">
+        <v>634.88818359375</v>
+      </c>
+      <c r="F20" t="n">
+        <v>20219900</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>45967</v>
+      </c>
+      <c r="B21" t="n">
+        <v>634.7882936522686</v>
+      </c>
+      <c r="C21" t="n">
+        <v>634.938067569805</v>
+      </c>
+      <c r="D21" t="n">
+        <v>616.9681222612256</v>
+      </c>
+      <c r="E21" t="n">
+        <v>617.9065551757812</v>
+      </c>
+      <c r="F21" t="n">
+        <v>23628800</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>45968</v>
+      </c>
+      <c r="B22" t="n">
+        <v>615.4606203242017</v>
+      </c>
+      <c r="C22" t="n">
+        <v>621.0912176885568</v>
+      </c>
+      <c r="D22" t="n">
+        <v>600.1961723842201</v>
+      </c>
+      <c r="E22" t="n">
+        <v>620.6719360351562</v>
+      </c>
+      <c r="F22" t="n">
+        <v>29946800</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>45971</v>
+      </c>
+      <c r="B23" t="n">
+        <v>630.0363359130761</v>
+      </c>
+      <c r="C23" t="n">
+        <v>633.9397808237388</v>
+      </c>
+      <c r="D23" t="n">
+        <v>617.077966360211</v>
+      </c>
+      <c r="E23" t="n">
+        <v>630.7052001953125</v>
+      </c>
+      <c r="F23" t="n">
+        <v>19245000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>45972</v>
+      </c>
+      <c r="B24" t="n">
+        <v>626.9514668906089</v>
+      </c>
+      <c r="C24" t="n">
+        <v>628.5088598168925</v>
+      </c>
+      <c r="D24" t="n">
+        <v>618.3558571038752</v>
+      </c>
+      <c r="E24" t="n">
+        <v>626.0330200195312</v>
+      </c>
+      <c r="F24" t="n">
+        <v>13302200</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>45973</v>
+      </c>
+      <c r="B25" t="n">
+        <v>627.0812350986922</v>
+      </c>
+      <c r="C25" t="n">
+        <v>627.939784558569</v>
+      </c>
+      <c r="D25" t="n">
+        <v>606.7552442025384</v>
+      </c>
+      <c r="E25" t="n">
+        <v>607.9931640625</v>
+      </c>
+      <c r="F25" t="n">
+        <v>24493300</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>45974</v>
+      </c>
+      <c r="B26" t="n">
+        <v>612.0463872625083</v>
+      </c>
+      <c r="C26" t="n">
+        <v>616.6187572691151</v>
+      </c>
+      <c r="D26" t="n">
+        <v>601.993193452889</v>
+      </c>
+      <c r="E26" t="n">
+        <v>608.8717041015625</v>
+      </c>
+      <c r="F26" t="n">
+        <v>20973800</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>45975</v>
+      </c>
+      <c r="B27" t="n">
+        <v>600.7852061056304</v>
+      </c>
+      <c r="C27" t="n">
+        <v>612.6553687237855</v>
+      </c>
+      <c r="D27" t="n">
+        <v>594.2062431482154</v>
+      </c>
+      <c r="E27" t="n">
+        <v>608.4424438476562</v>
+      </c>
+      <c r="F27" t="n">
+        <v>20724100</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>45978</v>
+      </c>
+      <c r="B28" t="n">
+        <v>608.0230519623859</v>
+      </c>
+      <c r="C28" t="n">
+        <v>610.6686515784111</v>
+      </c>
+      <c r="D28" t="n">
+        <v>594.4058732487083</v>
+      </c>
+      <c r="E28" t="n">
+        <v>601.0048217773438</v>
+      </c>
+      <c r="F28" t="n">
+        <v>16501300</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>45979</v>
+      </c>
+      <c r="B29" t="n">
+        <v>590.612218909938</v>
+      </c>
+      <c r="C29" t="n">
+        <v>602.6520806612418</v>
+      </c>
+      <c r="D29" t="n">
+        <v>582.8053290854997</v>
+      </c>
+      <c r="E29" t="n">
+        <v>596.6920776367188</v>
+      </c>
+      <c r="F29" t="n">
+        <v>25500600</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>45980</v>
+      </c>
+      <c r="B30" t="n">
+        <v>592.7286370493186</v>
+      </c>
+      <c r="C30" t="n">
+        <v>594.3359951431619</v>
+      </c>
+      <c r="D30" t="n">
+        <v>580.2794874440681</v>
+      </c>
+      <c r="E30" t="n">
+        <v>589.3343505859375</v>
+      </c>
+      <c r="F30" t="n">
+        <v>24744700</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>45981</v>
+      </c>
+      <c r="B31" t="n">
+        <v>602.4923362369276</v>
+      </c>
+      <c r="C31" t="n">
+        <v>605.706930555967</v>
+      </c>
+      <c r="D31" t="n">
+        <v>582.375956312388</v>
+      </c>
+      <c r="E31" t="n">
+        <v>588.1663208007812</v>
+      </c>
+      <c r="F31" t="n">
+        <v>20603000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>45982</v>
+      </c>
+      <c r="B32" t="n">
+        <v>587.517412968027</v>
+      </c>
+      <c r="C32" t="n">
+        <v>597.1213460929463</v>
+      </c>
+      <c r="D32" t="n">
+        <v>580.88848479756</v>
+      </c>
+      <c r="E32" t="n">
+        <v>593.2578125</v>
+      </c>
+      <c r="F32" t="n">
+        <v>21052600</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>45985</v>
+      </c>
+      <c r="B33" t="n">
+        <v>597.7203367937327</v>
+      </c>
+      <c r="C33" t="n">
+        <v>615.6703584886146</v>
+      </c>
+      <c r="D33" t="n">
+        <v>596.6321908004635</v>
+      </c>
+      <c r="E33" t="n">
+        <v>612.0264282226562</v>
+      </c>
+      <c r="F33" t="n">
+        <v>23554900</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>45986</v>
+      </c>
+      <c r="B34" t="n">
+        <v>622.9580871825591</v>
+      </c>
+      <c r="C34" t="n">
+        <v>635.9862849922763</v>
+      </c>
+      <c r="D34" t="n">
+        <v>617.2675924687619</v>
+      </c>
+      <c r="E34" t="n">
+        <v>635.1576538085938</v>
+      </c>
+      <c r="F34" t="n">
+        <v>25213000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>45987</v>
+      </c>
+      <c r="B35" t="n">
+        <v>636.6252677780955</v>
+      </c>
+      <c r="C35" t="n">
+        <v>637.2941320349476</v>
+      </c>
+      <c r="D35" t="n">
+        <v>630.5753884422047</v>
+      </c>
+      <c r="E35" t="n">
+        <v>632.5520629882812</v>
+      </c>
+      <c r="F35" t="n">
+        <v>15209500</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>45989</v>
+      </c>
+      <c r="B36" t="n">
+        <v>635.0179876534709</v>
+      </c>
+      <c r="C36" t="n">
+        <v>646.9679727244463</v>
+      </c>
+      <c r="D36" t="n">
+        <v>634.4389389877349</v>
+      </c>
+      <c r="E36" t="n">
+        <v>646.8681640625</v>
+      </c>
+      <c r="F36" t="n">
+        <v>11033200</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B37" t="n">
+        <v>638.4821234657416</v>
+      </c>
+      <c r="C37" t="n">
+        <v>644.2425087257971</v>
+      </c>
+      <c r="D37" t="n">
+        <v>636.6951341862962</v>
+      </c>
+      <c r="E37" t="n">
+        <v>639.7999267578125</v>
+      </c>
+      <c r="F37" t="n">
+        <v>13029900</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>45993</v>
+      </c>
+      <c r="B38" t="n">
+        <v>641.2675300698932</v>
+      </c>
+      <c r="C38" t="n">
+        <v>646.7882651016448</v>
+      </c>
+      <c r="D38" t="n">
+        <v>637.0046400682228</v>
+      </c>
+      <c r="E38" t="n">
+        <v>646.01953125</v>
+      </c>
+      <c r="F38" t="n">
+        <v>11640900</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>45994</v>
+      </c>
+      <c r="B39" t="n">
+        <v>643.3340098224904</v>
+      </c>
+      <c r="C39" t="n">
+        <v>647.7665988470103</v>
+      </c>
+      <c r="D39" t="n">
+        <v>636.4854785031988</v>
+      </c>
+      <c r="E39" t="n">
+        <v>638.5320434570312</v>
+      </c>
+      <c r="F39" t="n">
+        <v>11134300</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>45995</v>
+      </c>
+      <c r="B40" t="n">
+        <v>674.87134871331</v>
+      </c>
+      <c r="C40" t="n">
+        <v>674.9711573797597</v>
+      </c>
+      <c r="D40" t="n">
+        <v>658.9479666864565</v>
+      </c>
+      <c r="E40" t="n">
+        <v>660.425537109375</v>
+      </c>
+      <c r="F40" t="n">
+        <v>29874600</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>45996</v>
+      </c>
+      <c r="B41" t="n">
+        <v>662.8913386215002</v>
+      </c>
+      <c r="C41" t="n">
+        <v>673.5634922785046</v>
+      </c>
+      <c r="D41" t="n">
+        <v>661.2840414153883</v>
+      </c>
+      <c r="E41" t="n">
+        <v>672.2955932617188</v>
+      </c>
+      <c r="F41" t="n">
+        <v>21207900</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>45999</v>
+      </c>
+      <c r="B42" t="n">
+        <v>668.2224435191038</v>
+      </c>
+      <c r="C42" t="n">
+        <v>675.5801331063639</v>
+      </c>
+      <c r="D42" t="n">
+        <v>663.9595535520253</v>
+      </c>
+      <c r="E42" t="n">
+        <v>665.6866455078125</v>
+      </c>
+      <c r="F42" t="n">
+        <v>13161000</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>46000</v>
+      </c>
+      <c r="B43" t="n">
+        <v>662.6617867420982</v>
+      </c>
+      <c r="C43" t="n">
+        <v>663.3705623262879</v>
+      </c>
+      <c r="D43" t="n">
+        <v>652.2492080192432</v>
+      </c>
+      <c r="E43" t="n">
+        <v>655.8631591796875</v>
+      </c>
+      <c r="F43" t="n">
+        <v>12997100</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>46001</v>
+      </c>
+      <c r="B44" t="n">
+        <v>648.8648024836247</v>
+      </c>
+      <c r="C44" t="n">
+        <v>653.4171862971667</v>
+      </c>
+      <c r="D44" t="n">
+        <v>642.3257510862366</v>
+      </c>
+      <c r="E44" t="n">
+        <v>649.0444946289062</v>
+      </c>
+      <c r="F44" t="n">
+        <v>16910900</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
+        <v>46002</v>
+      </c>
+      <c r="B45" t="n">
+        <v>642.2158631242634</v>
+      </c>
+      <c r="C45" t="n">
+        <v>654.1858943512054</v>
+      </c>
+      <c r="D45" t="n">
+        <v>639.730030479328</v>
+      </c>
+      <c r="E45" t="n">
+        <v>651.6201782226562</v>
+      </c>
+      <c r="F45" t="n">
+        <v>13056700</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>46003</v>
+      </c>
+      <c r="B46" t="n">
+        <v>648.7150654102267</v>
+      </c>
+      <c r="C46" t="n">
+        <v>709.8128965395189</v>
+      </c>
+      <c r="D46" t="n">
+        <v>637.543746077992</v>
+      </c>
+      <c r="E46" t="n">
+        <v>643.1543579101562</v>
+      </c>
+      <c r="F46" t="n">
+        <v>14016900</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>46006</v>
+      </c>
+      <c r="B47" t="n">
+        <v>645.1476664750544</v>
+      </c>
+      <c r="C47" t="n">
+        <v>652.4414097008485</v>
+      </c>
+      <c r="D47" t="n">
+        <v>638.1536544261938</v>
+      </c>
+      <c r="E47" t="n">
+        <v>646.9561157226562</v>
+      </c>
+      <c r="F47" t="n">
+        <v>15549100</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>46007</v>
+      </c>
+      <c r="B48" t="n">
+        <v>642.9495426008936</v>
+      </c>
+      <c r="C48" t="n">
+        <v>661.973233609148</v>
+      </c>
+      <c r="D48" t="n">
+        <v>642.6498114209788</v>
+      </c>
+      <c r="E48" t="n">
+        <v>656.587890625</v>
+      </c>
+      <c r="F48" t="n">
+        <v>14309100</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
+        <v>46008</v>
+      </c>
+      <c r="B49" t="n">
+        <v>655.0491556477624</v>
+      </c>
+      <c r="C49" t="n">
+        <v>660.664343241777</v>
+      </c>
+      <c r="D49" t="n">
+        <v>648.644665798819</v>
+      </c>
+      <c r="E49" t="n">
+        <v>648.9443969726562</v>
+      </c>
+      <c r="F49" t="n">
+        <v>15598500</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="n">
+        <v>46009</v>
+      </c>
+      <c r="B50" t="n">
+        <v>656.4679564970005</v>
+      </c>
+      <c r="C50" t="n">
+        <v>669.9863502083882</v>
+      </c>
+      <c r="D50" t="n">
+        <v>655.8984367998282</v>
+      </c>
+      <c r="E50" t="n">
+        <v>663.881591796875</v>
+      </c>
+      <c r="F50" t="n">
+        <v>20260300</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="n">
+        <v>46010</v>
+      </c>
+      <c r="B51" t="n">
+        <v>665.8499012351181</v>
+      </c>
+      <c r="C51" t="n">
+        <v>670.4260003995075</v>
+      </c>
+      <c r="D51" t="n">
+        <v>657.6169598101359</v>
+      </c>
+      <c r="E51" t="n">
+        <v>658.2064819335938</v>
+      </c>
+      <c r="F51" t="n">
+        <v>49977100</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>46013</v>
+      </c>
+      <c r="B52" t="n">
+        <v>661.0840391473547</v>
+      </c>
+      <c r="C52" t="n">
+        <v>673.0038267300547</v>
+      </c>
+      <c r="D52" t="n">
+        <v>656.0883162216827</v>
+      </c>
+      <c r="E52" t="n">
+        <v>660.9341430664062</v>
+      </c>
+      <c r="F52" t="n">
+        <v>15659400</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="n">
+        <v>46014</v>
+      </c>
+      <c r="B53" t="n">
+        <v>659.4853234816244</v>
+      </c>
+      <c r="C53" t="n">
+        <v>665.4302455294139</v>
+      </c>
+      <c r="D53" t="n">
+        <v>657.6868755551602</v>
+      </c>
+      <c r="E53" t="n">
+        <v>664.3711547851562</v>
+      </c>
+      <c r="F53" t="n">
+        <v>8486800</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>46015</v>
+      </c>
+      <c r="B54" t="n">
+        <v>661.9632786179176</v>
+      </c>
+      <c r="C54" t="n">
+        <v>667.6084088263418</v>
+      </c>
+      <c r="D54" t="n">
+        <v>661.633543835896</v>
+      </c>
+      <c r="E54" t="n">
+        <v>666.9789428710938</v>
+      </c>
+      <c r="F54" t="n">
+        <v>5627500</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="n">
+        <v>46017</v>
+      </c>
+      <c r="B55" t="n">
+        <v>667.4885344385556</v>
+      </c>
+      <c r="C55" t="n">
+        <v>668.3777877623371</v>
+      </c>
+      <c r="D55" t="n">
+        <v>660.7543096382171</v>
+      </c>
+      <c r="E55" t="n">
+        <v>662.7225952148438</v>
+      </c>
+      <c r="F55" t="n">
+        <v>7133800</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>46020</v>
+      </c>
+      <c r="B56" t="n">
+        <v>657.4471149030659</v>
+      </c>
+      <c r="C56" t="n">
+        <v>659.6851889371151</v>
+      </c>
+      <c r="D56" t="n">
+        <v>653.8302165118</v>
+      </c>
+      <c r="E56" t="n">
+        <v>658.1265258789062</v>
+      </c>
+      <c r="F56" t="n">
+        <v>8506500</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n">
+        <v>46021</v>
+      </c>
+      <c r="B57" t="n">
+        <v>658.1265110341435</v>
+      </c>
+      <c r="C57" t="n">
+        <v>671.6449047754843</v>
+      </c>
+      <c r="D57" t="n">
+        <v>657.2772625792347</v>
+      </c>
+      <c r="E57" t="n">
+        <v>665.3803100585938</v>
+      </c>
+      <c r="F57" t="n">
+        <v>9187500</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>46022</v>
+      </c>
+      <c r="B58" t="n">
+        <v>664.1813161961976</v>
+      </c>
+      <c r="C58" t="n">
+        <v>664.4311023248911</v>
+      </c>
+      <c r="D58" t="n">
+        <v>658.8758612620638</v>
+      </c>
+      <c r="E58" t="n">
+        <v>659.5253295898438</v>
+      </c>
+      <c r="F58" t="n">
+        <v>7940400</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="n">
+        <v>46024</v>
+      </c>
+      <c r="B59" t="n">
+        <v>662.1630447721155</v>
+      </c>
+      <c r="C59" t="n">
+        <v>663.8216588672108</v>
+      </c>
+      <c r="D59" t="n">
+        <v>642.9495146869224</v>
+      </c>
+      <c r="E59" t="n">
+        <v>649.8535766601562</v>
+      </c>
+      <c r="F59" t="n">
+        <v>13726500</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B60" t="n">
+        <v>650.4531272549772</v>
+      </c>
+      <c r="C60" t="n">
+        <v>663.9715218041853</v>
+      </c>
+      <c r="D60" t="n">
+        <v>647.1959061445123</v>
+      </c>
+      <c r="E60" t="n">
+        <v>658.2264404296875</v>
+      </c>
+      <c r="F60" t="n">
+        <v>12213700</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n">
+        <v>46028</v>
+      </c>
+      <c r="B61" t="n">
+        <v>659.0057810200069</v>
+      </c>
+      <c r="C61" t="n">
+        <v>664.9507033148827</v>
+      </c>
+      <c r="D61" t="n">
+        <v>651.3423593634897</v>
+      </c>
+      <c r="E61" t="n">
+        <v>660.0548706054688</v>
+      </c>
+      <c r="F61" t="n">
+        <v>11074400</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="n">
+        <v>46029</v>
+      </c>
+      <c r="B62" t="n">
+        <v>655.0791375151089</v>
+      </c>
+      <c r="C62" t="n">
+        <v>658.5861445899717</v>
+      </c>
+      <c r="D62" t="n">
+        <v>644.2583851266311</v>
+      </c>
+      <c r="E62" t="n">
+        <v>648.1350708007812</v>
+      </c>
+      <c r="F62" t="n">
+        <v>12846300</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="n">
+        <v>46030</v>
+      </c>
+      <c r="B63" t="n">
+        <v>645.3274855180696</v>
+      </c>
+      <c r="C63" t="n">
+        <v>646.5464125947736</v>
+      </c>
+      <c r="D63" t="n">
+        <v>635.1761427603</v>
+      </c>
+      <c r="E63" t="n">
+        <v>645.50732421875</v>
+      </c>
+      <c r="F63" t="n">
+        <v>11921700</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="n">
+        <v>46031</v>
+      </c>
+      <c r="B64" t="n">
+        <v>644.8878661181845</v>
+      </c>
+      <c r="C64" t="n">
+        <v>654.3897406244424</v>
+      </c>
+      <c r="D64" t="n">
+        <v>642.3000548798136</v>
+      </c>
+      <c r="E64" t="n">
+        <v>652.5013427734375</v>
+      </c>
+      <c r="F64" t="n">
+        <v>11634900</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="n">
+        <v>46034</v>
+      </c>
+      <c r="B65" t="n">
+        <v>651.9718010113269</v>
+      </c>
+      <c r="C65" t="n">
+        <v>653.4105105723186</v>
+      </c>
+      <c r="D65" t="n">
+        <v>640.6814191818085</v>
+      </c>
+      <c r="E65" t="n">
+        <v>641.4207763671875</v>
+      </c>
+      <c r="F65" t="n">
+        <v>14797200</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="n">
+        <v>46035</v>
+      </c>
+      <c r="B66" t="n">
+        <v>641.720599826752</v>
+      </c>
+      <c r="C66" t="n">
+        <v>641.720599826752</v>
+      </c>
+      <c r="D66" t="n">
+        <v>623.5660991574318</v>
+      </c>
+      <c r="E66" t="n">
+        <v>630.5501708984375</v>
+      </c>
+      <c r="F66" t="n">
+        <v>18030400</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="n">
+        <v>46036</v>
+      </c>
+      <c r="B67" t="n">
+        <v>625.9640568168747</v>
+      </c>
+      <c r="C67" t="n">
+        <v>627.9124008742662</v>
+      </c>
+      <c r="D67" t="n">
+        <v>614.2940558608916</v>
+      </c>
+      <c r="E67" t="n">
+        <v>614.9934692382812</v>
+      </c>
+      <c r="F67" t="n">
+        <v>15527900</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="n">
+        <v>46037</v>
+      </c>
+      <c r="B68" t="n">
+        <v>617.9508982377323</v>
+      </c>
+      <c r="C68" t="n">
+        <v>623.6360331340583</v>
+      </c>
+      <c r="D68" t="n">
+        <v>613.7045339245012</v>
+      </c>
+      <c r="E68" t="n">
+        <v>620.2689208984375</v>
+      </c>
+      <c r="F68" t="n">
+        <v>13076100</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="n">
+        <v>46038</v>
+      </c>
+      <c r="B69" t="n">
+        <v>623.6460522405506</v>
+      </c>
+      <c r="C69" t="n">
+        <v>628.5418850412981</v>
+      </c>
+      <c r="D69" t="n">
+        <v>619.5495838845379</v>
+      </c>
+      <c r="E69" t="n">
+        <v>619.7194213867188</v>
+      </c>
+      <c r="F69" t="n">
+        <v>17012500</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="n">
+        <v>46042</v>
+      </c>
+      <c r="B70" t="n">
+        <v>607.3600037753715</v>
+      </c>
+      <c r="C70" t="n">
+        <v>610.8770121629093</v>
+      </c>
+      <c r="D70" t="n">
+        <v>599.4867397151437</v>
+      </c>
+      <c r="E70" t="n">
+        <v>603.6032104492188</v>
+      </c>
+      <c r="F70" t="n">
+        <v>15169600</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="n">
+        <v>46043</v>
+      </c>
+      <c r="B71" t="n">
+        <v>606.2209580964126</v>
+      </c>
+      <c r="C71" t="n">
+        <v>617.7411240978843</v>
+      </c>
+      <c r="D71" t="n">
+        <v>599.5666821865381</v>
+      </c>
+      <c r="E71" t="n">
+        <v>612.4356689453125</v>
+      </c>
+      <c r="F71" t="n">
+        <v>14494700</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B72" t="n">
+        <v>628.811597152667</v>
+      </c>
+      <c r="C72" t="n">
+        <v>660.0049216653568</v>
+      </c>
+      <c r="D72" t="n">
+        <v>626.0140046136898</v>
+      </c>
+      <c r="E72" t="n">
+        <v>647.0759887695312</v>
+      </c>
+      <c r="F72" t="n">
+        <v>21394700</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="n">
+        <v>46045</v>
+      </c>
+      <c r="B73" t="n">
+        <v>644.2184496993522</v>
+      </c>
+      <c r="C73" t="n">
+        <v>665.9198400091174</v>
+      </c>
+      <c r="D73" t="n">
+        <v>643.8987161260534</v>
+      </c>
+      <c r="E73" t="n">
+        <v>658.1964721679688</v>
+      </c>
+      <c r="F73" t="n">
+        <v>22797700</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="n">
+        <v>46048</v>
+      </c>
+      <c r="B74" t="n">
+        <v>664.5609947255355</v>
+      </c>
+      <c r="C74" t="n">
+        <v>674.7023359243682</v>
+      </c>
+      <c r="D74" t="n">
+        <v>660.7242529636108</v>
+      </c>
+      <c r="E74" t="n">
+        <v>671.7847900390625</v>
+      </c>
+      <c r="F74" t="n">
+        <v>16327400</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="n">
+        <v>46049</v>
+      </c>
+      <c r="B75" t="n">
+        <v>674.0129574053085</v>
+      </c>
+      <c r="C75" t="n">
+        <v>676.2410302656567</v>
+      </c>
+      <c r="D75" t="n">
+        <v>664.0913982323968</v>
+      </c>
+      <c r="E75" t="n">
+        <v>672.394287109375</v>
+      </c>
+      <c r="F75" t="n">
+        <v>13297400</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="n">
+        <v>46050</v>
+      </c>
+      <c r="B76" t="n">
+        <v>673.9229813666298</v>
+      </c>
+      <c r="C76" t="n">
+        <v>677.1002536346601</v>
+      </c>
+      <c r="D76" t="n">
+        <v>665.5301429727417</v>
+      </c>
+      <c r="E76" t="n">
+        <v>668.1578979492188</v>
+      </c>
+      <c r="F76" t="n">
+        <v>25709600</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="n">
+        <v>46051</v>
+      </c>
+      <c r="B77" t="n">
+        <v>736.7991536844581</v>
+      </c>
+      <c r="C77" t="n">
+        <v>743.363540655783</v>
+      </c>
+      <c r="D77" t="n">
+        <v>711.9404325537852</v>
+      </c>
+      <c r="E77" t="n">
+        <v>737.6784057617188</v>
+      </c>
+      <c r="F77" t="n">
+        <v>59852900</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="n">
+        <v>46052</v>
+      </c>
+      <c r="B78" t="n">
+        <v>726.8776752394725</v>
+      </c>
+      <c r="C78" t="n">
+        <v>731.5436633097714</v>
+      </c>
+      <c r="D78" t="n">
+        <v>712.9796010924755</v>
+      </c>
+      <c r="E78" t="n">
+        <v>715.8870849609375</v>
+      </c>
+      <c r="F78" t="n">
+        <v>23744600</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B79" t="n">
+        <v>713.9886602426056</v>
+      </c>
+      <c r="C79" t="n">
+        <v>720.6829408229889</v>
+      </c>
+      <c r="D79" t="n">
+        <v>702.9181827036907</v>
+      </c>
+      <c r="E79" t="n">
+        <v>705.8056640625</v>
+      </c>
+      <c r="F79" t="n">
+        <v>14365200</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="n">
+        <v>46056</v>
+      </c>
+      <c r="B80" t="n">
+        <v>706.7648539132639</v>
+      </c>
+      <c r="C80" t="n">
+        <v>716.3866205151361</v>
+      </c>
+      <c r="D80" t="n">
+        <v>685.8227628297016</v>
+      </c>
+      <c r="E80" t="n">
+        <v>691.1082763671875</v>
+      </c>
+      <c r="F80" t="n">
+        <v>13760700</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="n">
+        <v>46057</v>
+      </c>
+      <c r="B81" t="n">
+        <v>687.1416843315144</v>
+      </c>
+      <c r="C81" t="n">
+        <v>688.2407799622291</v>
+      </c>
+      <c r="D81" t="n">
+        <v>666.8890651090074</v>
+      </c>
+      <c r="E81" t="n">
+        <v>668.417724609375</v>
+      </c>
+      <c r="F81" t="n">
+        <v>16882800</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="n">
+        <v>46058</v>
+      </c>
+      <c r="B82" t="n">
+        <v>663.0123852284637</v>
+      </c>
+      <c r="C82" t="n">
+        <v>680.9170392363125</v>
+      </c>
+      <c r="D82" t="n">
+        <v>652.9409906690098</v>
+      </c>
+      <c r="E82" t="n">
+        <v>669.63671875</v>
+      </c>
+      <c r="F82" t="n">
+        <v>17131800</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B83" t="n">
+        <v>664.920685797671</v>
+      </c>
+      <c r="C83" t="n">
+        <v>671.4151252649915</v>
+      </c>
+      <c r="D83" t="n">
+        <v>645.9469408650316</v>
+      </c>
+      <c r="E83" t="n">
+        <v>660.8941650390625</v>
+      </c>
+      <c r="F83" t="n">
+        <v>18159300</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B84" t="n">
+        <v>662.6126578425271</v>
+      </c>
+      <c r="C84" t="n">
+        <v>682.7254419812133</v>
+      </c>
+      <c r="D84" t="n">
+        <v>658.2164585284562</v>
+      </c>
+      <c r="E84" t="n">
+        <v>676.640625</v>
+      </c>
+      <c r="F84" t="n">
+        <v>14837500</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="n">
+        <v>46063</v>
+      </c>
+      <c r="B85" t="n">
+        <v>677.0202983345941</v>
+      </c>
+      <c r="C85" t="n">
+        <v>680.0677378888336</v>
+      </c>
+      <c r="D85" t="n">
+        <v>669.216982119095</v>
+      </c>
+      <c r="E85" t="n">
+        <v>670.1461791992188</v>
+      </c>
+      <c r="F85" t="n">
+        <v>10455800</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="n">
+        <v>46064</v>
+      </c>
+      <c r="B86" t="n">
+        <v>673.4234361526849</v>
+      </c>
+      <c r="C86" t="n">
+        <v>678.6889475196376</v>
+      </c>
+      <c r="D86" t="n">
+        <v>656.5378686274887</v>
+      </c>
+      <c r="E86" t="n">
+        <v>668.1179809570312</v>
+      </c>
+      <c r="F86" t="n">
+        <v>14323800</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="n">
+        <v>46065</v>
+      </c>
+      <c r="B87" t="n">
+        <v>669.3968787035581</v>
+      </c>
+      <c r="C87" t="n">
+        <v>675.421749916193</v>
+      </c>
+      <c r="D87" t="n">
+        <v>644.7280570616384</v>
+      </c>
+      <c r="E87" t="n">
+        <v>649.254150390625</v>
+      </c>
+      <c r="F87" t="n">
+        <v>14960100</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="n">
+        <v>46066</v>
+      </c>
+      <c r="B88" t="n">
+        <v>644.5481137374378</v>
+      </c>
+      <c r="C88" t="n">
+        <v>650.872715705495</v>
+      </c>
+      <c r="D88" t="n">
+        <v>634.0271535178357</v>
+      </c>
+      <c r="E88" t="n">
+        <v>639.2227172851562</v>
+      </c>
+      <c r="F88" t="n">
+        <v>12336400</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="n">
+        <v>46070</v>
+      </c>
+      <c r="B89" t="n">
+        <v>638.952945338547</v>
+      </c>
+      <c r="C89" t="n">
+        <v>642.0502690775812</v>
+      </c>
+      <c r="D89" t="n">
+        <v>628.2620863630333</v>
+      </c>
+      <c r="E89" t="n">
+        <v>638.7431030273438</v>
+      </c>
+      <c r="F89" t="n">
+        <v>12674700</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="n">
+        <v>46071</v>
+      </c>
+      <c r="B90" t="n">
+        <v>633.2578140286595</v>
+      </c>
+      <c r="C90" t="n">
+        <v>644.4482453696517</v>
+      </c>
+      <c r="D90" t="n">
+        <v>627.6126838179015</v>
+      </c>
+      <c r="E90" t="n">
+        <v>642.6697387695312</v>
+      </c>
+      <c r="F90" t="n">
+        <v>14649200</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="n">
+        <v>46072</v>
+      </c>
+      <c r="B91" t="n">
+        <v>638.0237449576674</v>
+      </c>
+      <c r="C91" t="n">
+        <v>646.6363661317032</v>
+      </c>
+      <c r="D91" t="n">
+        <v>636.1752909436037</v>
+      </c>
+      <c r="E91" t="n">
+        <v>644.2284545898438</v>
+      </c>
+      <c r="F91" t="n">
+        <v>10035700</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="n">
+        <v>46073</v>
+      </c>
+      <c r="B92" t="n">
+        <v>639.1428111159805</v>
+      </c>
+      <c r="C92" t="n">
+        <v>662.7825455010891</v>
+      </c>
+      <c r="D92" t="n">
+        <v>638.2336163631846</v>
+      </c>
+      <c r="E92" t="n">
+        <v>655.09912109375</v>
+      </c>
+      <c r="F92" t="n">
+        <v>14183500</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="n">
+        <v>46076</v>
+      </c>
+      <c r="B93" t="n">
+        <v>651.9817939677475</v>
+      </c>
+      <c r="C93" t="n">
+        <v>657.1374142434245</v>
+      </c>
+      <c r="D93" t="n">
+        <v>635.455964272141</v>
+      </c>
+      <c r="E93" t="n">
+        <v>636.7048950195312</v>
+      </c>
+      <c r="F93" t="n">
+        <v>8605900</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="n">
+        <v>46077</v>
+      </c>
+      <c r="B94" t="n">
+        <v>632.5384628258726</v>
+      </c>
+      <c r="C94" t="n">
+        <v>640.5615620292823</v>
+      </c>
+      <c r="D94" t="n">
+        <v>628.4419334902003</v>
+      </c>
+      <c r="E94" t="n">
+        <v>638.7531127929688</v>
+      </c>
+      <c r="F94" t="n">
+        <v>10135600</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="n">
+        <v>46078</v>
+      </c>
+      <c r="B95" t="n">
+        <v>641.9803720795121</v>
+      </c>
+      <c r="C95" t="n">
+        <v>653.3206382422114</v>
+      </c>
+      <c r="D95" t="n">
+        <v>641.5906910720822</v>
+      </c>
+      <c r="E95" t="n">
+        <v>653.1307983398438</v>
+      </c>
+      <c r="F95" t="n">
+        <v>11330700</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="n">
+        <v>46079</v>
+      </c>
+      <c r="B96" t="n">
+        <v>649.9935020296807</v>
+      </c>
+      <c r="C96" t="n">
+        <v>660.4345752110744</v>
+      </c>
+      <c r="D96" t="n">
+        <v>646.9461232211356</v>
+      </c>
+      <c r="E96" t="n">
+        <v>656.447998046875</v>
+      </c>
+      <c r="F96" t="n">
+        <v>10637700</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="n">
+        <v>46080</v>
+      </c>
+      <c r="B97" t="n">
+        <v>642.8995542116262</v>
+      </c>
+      <c r="C97" t="n">
+        <v>648.8844201349368</v>
+      </c>
+      <c r="D97" t="n">
+        <v>637.5740968396581</v>
+      </c>
+      <c r="E97" t="n">
+        <v>647.62548828125</v>
+      </c>
+      <c r="F97" t="n">
+        <v>15703000</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B98" t="n">
+        <v>636.6149203669017</v>
+      </c>
+      <c r="C98" t="n">
+        <v>659.3754626922687</v>
+      </c>
+      <c r="D98" t="n">
+        <v>633.9572226725116</v>
+      </c>
+      <c r="E98" t="n">
+        <v>653.0009155273438</v>
+      </c>
+      <c r="F98" t="n">
+        <v>9816100</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="n">
+        <v>46084</v>
+      </c>
+      <c r="B99" t="n">
+        <v>647.7354225434952</v>
+      </c>
+      <c r="C99" t="n">
+        <v>658.4762268569145</v>
+      </c>
+      <c r="D99" t="n">
+        <v>638.2935549799161</v>
+      </c>
+      <c r="E99" t="n">
+        <v>654.5196533203125</v>
+      </c>
+      <c r="F99" t="n">
+        <v>12263800</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="n">
+        <v>46085</v>
+      </c>
+      <c r="B100" t="n">
+        <v>657.397151925757</v>
+      </c>
+      <c r="C100" t="n">
+        <v>672.1944798634893</v>
+      </c>
+      <c r="D100" t="n">
+        <v>657.1073609851721</v>
+      </c>
+      <c r="E100" t="n">
+        <v>667.1587524414062</v>
+      </c>
+      <c r="F100" t="n">
+        <v>10810100</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="n">
+        <v>46086</v>
+      </c>
+      <c r="B101" t="n">
+        <v>661.363765843265</v>
+      </c>
+      <c r="C101" t="n">
+        <v>670.1262833419206</v>
+      </c>
+      <c r="D101" t="n">
+        <v>649.7537106790966</v>
+      </c>
+      <c r="E101" t="n">
+        <v>660.0049438476562</v>
+      </c>
+      <c r="F101" t="n">
+        <v>13341400</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="n">
+        <v>46087</v>
+      </c>
+      <c r="B102" t="n">
+        <v>647.3457881163396</v>
+      </c>
+      <c r="C102" t="n">
+        <v>648.9143914185428</v>
+      </c>
+      <c r="D102" t="n">
+        <v>635.5658346648192</v>
+      </c>
+      <c r="E102" t="n">
+        <v>644.308349609375</v>
+      </c>
+      <c r="F102" t="n">
+        <v>13159400</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B103" t="n">
+        <v>634.2369839533108</v>
+      </c>
+      <c r="C103" t="n">
+        <v>647.195859029807</v>
+      </c>
+      <c r="D103" t="n">
+        <v>626.2438278402449</v>
+      </c>
+      <c r="E103" t="n">
+        <v>646.836181640625</v>
+      </c>
+      <c r="F103" t="n">
+        <v>13489700</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="n">
+        <v>46091</v>
+      </c>
+      <c r="B104" t="n">
+        <v>653.0009245574777</v>
+      </c>
+      <c r="C104" t="n">
+        <v>659.7351492208539</v>
+      </c>
+      <c r="D104" t="n">
+        <v>648.444827744844</v>
+      </c>
+      <c r="E104" t="n">
+        <v>653.510498046875</v>
+      </c>
+      <c r="F104" t="n">
+        <v>9859300</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="n">
+        <v>46092</v>
+      </c>
+      <c r="B105" t="n">
+        <v>654.1999146227295</v>
+      </c>
+      <c r="C105" t="n">
+        <v>658.5561703533895</v>
+      </c>
+      <c r="D105" t="n">
+        <v>647.8053649208291</v>
+      </c>
+      <c r="E105" t="n">
+        <v>654.2998046875</v>
+      </c>
+      <c r="F105" t="n">
+        <v>8977200</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="B106" t="n">
+        <v>648.1950599902964</v>
+      </c>
+      <c r="C106" t="n">
+        <v>652.9409968457168</v>
+      </c>
+      <c r="D106" t="n">
+        <v>636.355220859953</v>
+      </c>
+      <c r="E106" t="n">
+        <v>637.6340942382812</v>
+      </c>
+      <c r="F106" t="n">
+        <v>11617500</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="n">
+        <v>46094</v>
+      </c>
+      <c r="B107" t="n">
+        <v>623.3562813254467</v>
+      </c>
+      <c r="C107" t="n">
+        <v>628.6317326131165</v>
+      </c>
+      <c r="D107" t="n">
+        <v>609.0285222575777</v>
+      </c>
+      <c r="E107" t="n">
+        <v>613.1849975585938</v>
+      </c>
+      <c r="F107" t="n">
+        <v>18957600</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B108" t="n">
+        <v>632</v>
+      </c>
+      <c r="C108" t="n">
+        <v>634.75</v>
+      </c>
+      <c r="D108" t="n">
+        <v>623.0999755859375</v>
+      </c>
+      <c r="E108" t="n">
+        <v>627.4500122070312</v>
+      </c>
+      <c r="F108" t="n">
+        <v>15134900</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B109" t="n">
+        <v>627.989990234375</v>
+      </c>
+      <c r="C109" t="n">
+        <v>636.5499877929688</v>
+      </c>
+      <c r="D109" t="n">
+        <v>621.7000122070312</v>
+      </c>
+      <c r="E109" t="n">
+        <v>622.6599731445312</v>
+      </c>
+      <c r="F109" t="n">
+        <v>10348800</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="n">
+        <v>46099</v>
+      </c>
+      <c r="B110" t="n">
+        <v>616.3400268554688</v>
+      </c>
+      <c r="C110" t="n">
+        <v>622.6500244140625</v>
+      </c>
+      <c r="D110" t="n">
+        <v>614.6099853515625</v>
+      </c>
+      <c r="E110" t="n">
+        <v>615.6799926757812</v>
+      </c>
+      <c r="F110" t="n">
+        <v>11726300</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="n">
+        <v>46100</v>
+      </c>
+      <c r="B111" t="n">
+        <v>612.1500244140625</v>
+      </c>
+      <c r="C111" t="n">
+        <v>613</v>
+      </c>
+      <c r="D111" t="n">
+        <v>602.260009765625</v>
+      </c>
+      <c r="E111" t="n">
+        <v>606.7000122070312</v>
+      </c>
+      <c r="F111" t="n">
+        <v>13247700</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="n">
+        <v>46101</v>
+      </c>
+      <c r="B112" t="n">
+        <v>603.530029296875</v>
+      </c>
+      <c r="C112" t="n">
+        <v>603.9600219726562</v>
+      </c>
+      <c r="D112" t="n">
+        <v>587.25</v>
+      </c>
+      <c r="E112" t="n">
+        <v>593.6599731445312</v>
+      </c>
+      <c r="F112" t="n">
+        <v>21214900</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="n">
+        <v>46104</v>
+      </c>
+      <c r="B113" t="n">
+        <v>605.7899780273438</v>
+      </c>
+      <c r="C113" t="n">
+        <v>608.6400146484375</v>
+      </c>
+      <c r="D113" t="n">
+        <v>599.010009765625</v>
+      </c>
+      <c r="E113" t="n">
+        <v>604.0599975585938</v>
+      </c>
+      <c r="F113" t="n">
+        <v>13638000</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="n">
+        <v>46105</v>
+      </c>
+      <c r="B114" t="n">
+        <v>599.0999755859375</v>
+      </c>
+      <c r="C114" t="n">
+        <v>601</v>
+      </c>
+      <c r="D114" t="n">
+        <v>591</v>
+      </c>
+      <c r="E114" t="n">
+        <v>592.9199829101562</v>
+      </c>
+      <c r="F114" t="n">
+        <v>10739700</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="n">
+        <v>46106</v>
+      </c>
+      <c r="B115" t="n">
+        <v>598.739990234375</v>
+      </c>
+      <c r="C115" t="n">
+        <v>603.6699829101562</v>
+      </c>
+      <c r="D115" t="n">
+        <v>593.4000244140625</v>
+      </c>
+      <c r="E115" t="n">
+        <v>594.8900146484375</v>
+      </c>
+      <c r="F115" t="n">
+        <v>12585000</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B116" t="n">
+        <v>582.489990234375</v>
+      </c>
+      <c r="C116" t="n">
+        <v>583</v>
+      </c>
+      <c r="D116" t="n">
+        <v>543.3499755859375</v>
+      </c>
+      <c r="E116" t="n">
+        <v>547.5399780273438</v>
+      </c>
+      <c r="F116" t="n">
+        <v>35780100</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="n">
+        <v>46108</v>
+      </c>
+      <c r="B117" t="n">
+        <v>540.0999755859375</v>
+      </c>
+      <c r="C117" t="n">
+        <v>543.5999755859375</v>
+      </c>
+      <c r="D117" t="n">
+        <v>520.260009765625</v>
+      </c>
+      <c r="E117" t="n">
+        <v>525.719970703125</v>
+      </c>
+      <c r="F117" t="n">
+        <v>30133000</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="n">
+        <v>46111</v>
+      </c>
+      <c r="B118" t="n">
+        <v>536.3800048828125</v>
+      </c>
+      <c r="C118" t="n">
+        <v>539.5499877929688</v>
+      </c>
+      <c r="D118" t="n">
+        <v>528.5399780273438</v>
+      </c>
+      <c r="E118" t="n">
+        <v>536.3800048828125</v>
+      </c>
+      <c r="F118" t="n">
+        <v>22795200</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B119" t="n">
+        <v>549.97998046875</v>
+      </c>
+      <c r="C119" t="n">
+        <v>573.6900024414062</v>
+      </c>
+      <c r="D119" t="n">
+        <v>546.77001953125</v>
+      </c>
+      <c r="E119" t="n">
+        <v>572.1300048828125</v>
+      </c>
+      <c r="F119" t="n">
+        <v>32898300</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B120" t="n">
+        <v>580.1300048828125</v>
+      </c>
+      <c r="C120" t="n">
+        <v>592.5499877929688</v>
+      </c>
+      <c r="D120" t="n">
+        <v>573.8200073242188</v>
+      </c>
+      <c r="E120" t="n">
+        <v>579.22998046875</v>
+      </c>
+      <c r="F120" t="n">
+        <v>23608100</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B121" t="n">
+        <v>566.0399780273438</v>
+      </c>
+      <c r="C121" t="n">
+        <v>578.5</v>
+      </c>
+      <c r="D121" t="n">
+        <v>559.7000122070312</v>
+      </c>
+      <c r="E121" t="n">
+        <v>574.4600219726562</v>
+      </c>
+      <c r="F121" t="n">
+        <v>13518500</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B122" t="n">
+        <v>577.6900024414062</v>
+      </c>
+      <c r="C122" t="n">
+        <v>582.7899780273438</v>
+      </c>
+      <c r="D122" t="n">
+        <v>572</v>
+      </c>
+      <c r="E122" t="n">
+        <v>573.02001953125</v>
+      </c>
+      <c r="F122" t="n">
+        <v>9489600</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="n">
+        <v>46119</v>
+      </c>
+      <c r="B123" t="n">
+        <v>571.9000244140625</v>
+      </c>
+      <c r="C123" t="n">
+        <v>572.9600219726562</v>
+      </c>
+      <c r="D123" t="n">
+        <v>564.760009765625</v>
+      </c>
+      <c r="E123" t="n">
+        <v>569.530029296875</v>
+      </c>
+      <c r="F123" t="n">
+        <v>5218536</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>